<commit_message>
Fix substring matching bug: isolate 原夢 (1 unit), 原夢六期 (13 units), and 小國民原夢 (31 units)
</commit_message>
<xml_diff>
--- a/宜蘭建案實價登錄銷售統計.xlsx
+++ b/宜蘭建案實價登錄銷售統計.xlsx
@@ -558,25 +558,25 @@
         <v>7</v>
       </c>
       <c r="F3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G3" t="str">
-        <v>85.7% (6/7戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H3" t="str">
-        <v>85.7%</v>
+        <v>100%</v>
       </c>
       <c r="I3">
-        <v>24.2</v>
+        <v>26.1</v>
       </c>
       <c r="J3" t="str">
-        <v>22.6 ~ 25.8</v>
+        <v>22.3 ~ 36.8</v>
       </c>
       <c r="K3">
-        <v>1849.3</v>
+        <v>1058</v>
       </c>
       <c r="L3" t="str">
-        <v>112/05/08</v>
+        <v>113/03/02</v>
       </c>
       <c r="M3">
         <v>10</v>
@@ -1410,25 +1410,25 @@
         <v>39</v>
       </c>
       <c r="F15">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="G15" t="str">
-        <v>89.7% (35/39戶)</v>
+        <v>76.9% (30/39戶)</v>
       </c>
       <c r="H15" t="str">
-        <v>89.7%</v>
+        <v>76.9%</v>
       </c>
       <c r="I15">
-        <v>19.8</v>
+        <v>18.8</v>
       </c>
       <c r="J15" t="str">
-        <v>17.8 ~ 24.5</v>
+        <v>17.8 ~ 19.7</v>
       </c>
       <c r="K15">
-        <v>655.6</v>
+        <v>468.6</v>
       </c>
       <c r="L15" t="str">
-        <v>112/05/26</v>
+        <v>110/12/25</v>
       </c>
       <c r="M15">
         <v>10</v>
@@ -2049,25 +2049,25 @@
         <v>21</v>
       </c>
       <c r="F24">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G24" t="str">
-        <v>85.7% (18/21戶)</v>
+        <v>66.7% (14/21戶)</v>
       </c>
       <c r="H24" t="str">
-        <v>85.7%</v>
+        <v>66.7%</v>
       </c>
       <c r="I24">
-        <v>26.6</v>
+        <v>24.8</v>
       </c>
       <c r="J24" t="str">
-        <v>21.6 ~ 36.2</v>
+        <v>21.6 ~ 27</v>
       </c>
       <c r="K24">
-        <v>1407.7</v>
+        <v>1329.9</v>
       </c>
       <c r="L24" t="str">
-        <v>113/03/26</v>
+        <v>113/03/16</v>
       </c>
       <c r="M24" t="str">
         <v>--</v>
@@ -2191,25 +2191,25 @@
         <v>28</v>
       </c>
       <c r="F26">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="G26" t="str">
-        <v>完銷 100%</v>
+        <v>78.6% (22/28戶)</v>
       </c>
       <c r="H26" t="str">
-        <v>100%</v>
+        <v>78.6%</v>
       </c>
       <c r="I26">
-        <v>20.9</v>
+        <v>20.4</v>
       </c>
       <c r="J26" t="str">
         <v>18.8 ~ 25.3</v>
       </c>
       <c r="K26">
-        <v>365.6</v>
+        <v>352.4</v>
       </c>
       <c r="L26" t="str">
-        <v>113/04/13</v>
+        <v>112/08/11</v>
       </c>
       <c r="M26" t="str">
         <v>--</v>
@@ -2262,25 +2262,25 @@
         <v>20</v>
       </c>
       <c r="F27">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G27" t="str">
-        <v>完銷 100%</v>
+        <v>80% (16/20戶)</v>
       </c>
       <c r="H27" t="str">
-        <v>100%</v>
+        <v>80%</v>
       </c>
       <c r="I27">
-        <v>29.5</v>
+        <v>25.3</v>
       </c>
       <c r="J27" t="str">
-        <v>21 ~ 40.3</v>
+        <v>21 ~ 30.4</v>
       </c>
       <c r="K27">
-        <v>785.7</v>
+        <v>799.6</v>
       </c>
       <c r="L27" t="str">
-        <v>113/12/20</v>
+        <v>111/03/05</v>
       </c>
       <c r="M27" t="str">
         <v>--</v>
@@ -2484,16 +2484,16 @@
         <v>100%</v>
       </c>
       <c r="I30">
-        <v>26.8</v>
+        <v>21.1</v>
       </c>
       <c r="J30" t="str">
-        <v>21.1 ~ 32.1</v>
+        <v>21.1 ~ 21.1</v>
       </c>
       <c r="K30">
-        <v>614</v>
+        <v>900</v>
       </c>
       <c r="L30" t="str">
-        <v>115/03/11</v>
+        <v>111/01/03</v>
       </c>
       <c r="M30">
         <v>8.7</v>
@@ -3123,16 +3123,16 @@
         <v>100%</v>
       </c>
       <c r="I39">
-        <v>18.8</v>
+        <v>17.7</v>
       </c>
       <c r="J39" t="str">
-        <v>17.7 ~ 19.3</v>
+        <v>13.8 ~ 19.3</v>
       </c>
       <c r="K39">
-        <v>835.8</v>
+        <v>744.1</v>
       </c>
       <c r="L39" t="str">
-        <v>111/06/12</v>
+        <v>111/09/05</v>
       </c>
       <c r="M39" t="str">
         <v>--</v>
@@ -3327,25 +3327,25 @@
         <v>10</v>
       </c>
       <c r="F42">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G42" t="str">
-        <v>80% (8/10戶)</v>
+        <v>50% (5/10戶)</v>
       </c>
       <c r="H42" t="str">
-        <v>80%</v>
+        <v>50%</v>
       </c>
       <c r="I42">
-        <v>22.6</v>
+        <v>22</v>
       </c>
       <c r="J42" t="str">
-        <v>21.3 ~ 26.9</v>
+        <v>21.3 ~ 22.6</v>
       </c>
       <c r="K42">
-        <v>1271.9</v>
+        <v>1275.3</v>
       </c>
       <c r="L42" t="str">
-        <v>113/12/10</v>
+        <v>112/05/27</v>
       </c>
       <c r="M42" t="str">
         <v>--</v>
@@ -5173,22 +5173,22 @@
         <v>16</v>
       </c>
       <c r="F68">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G68" t="str">
-        <v>31.3% (5/16戶)</v>
+        <v>37.5% (6/16戶)</v>
       </c>
       <c r="H68" t="str">
-        <v>31.3%</v>
+        <v>37.5%</v>
       </c>
       <c r="I68">
-        <v>20.2</v>
+        <v>20</v>
       </c>
       <c r="J68" t="str">
-        <v>17.8 ~ 21.8</v>
+        <v>17 ~ 21.8</v>
       </c>
       <c r="K68">
-        <v>838.7</v>
+        <v>843.8</v>
       </c>
       <c r="L68" t="str">
         <v>111/07/31</v>
@@ -5741,22 +5741,22 @@
         <v>48</v>
       </c>
       <c r="F76">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="G76" t="str">
-        <v>68.8% (33/48戶)</v>
+        <v>87.5% (42/48戶)</v>
       </c>
       <c r="H76" t="str">
-        <v>68.8%</v>
+        <v>87.5%</v>
       </c>
       <c r="I76">
-        <v>24.1</v>
+        <v>23</v>
       </c>
       <c r="J76" t="str">
-        <v>22.6 ~ 26.3</v>
+        <v>18 ~ 26.3</v>
       </c>
       <c r="K76">
-        <v>718.1</v>
+        <v>820.7</v>
       </c>
       <c r="L76" t="str">
         <v>113/03/26</v>
@@ -5883,22 +5883,22 @@
         <v>6</v>
       </c>
       <c r="F78">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G78" t="str">
-        <v>83.3% (5/6戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H78" t="str">
-        <v>83.3%</v>
+        <v>100%</v>
       </c>
       <c r="I78">
-        <v>20.5</v>
+        <v>19.6</v>
       </c>
       <c r="J78" t="str">
-        <v>20.4 ~ 21.2</v>
+        <v>18 ~ 21.2</v>
       </c>
       <c r="K78">
-        <v>1269.3</v>
+        <v>1201.8</v>
       </c>
       <c r="L78" t="str">
         <v>111/05/28</v>
@@ -7303,25 +7303,25 @@
         <v>7</v>
       </c>
       <c r="F98">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G98" t="str">
-        <v>完銷 100%</v>
+        <v>57.1% (4/7戶)</v>
       </c>
       <c r="H98" t="str">
-        <v>100%</v>
+        <v>57.1%</v>
       </c>
       <c r="I98">
-        <v>16.3</v>
+        <v>16.8</v>
       </c>
       <c r="J98" t="str">
-        <v>15.8 ~ 18.3</v>
+        <v>16.1 ~ 18.3</v>
       </c>
       <c r="K98">
-        <v>635.5</v>
+        <v>1024.6</v>
       </c>
       <c r="L98" t="str">
-        <v>113/01/16</v>
+        <v>111/09/21</v>
       </c>
       <c r="M98" t="str">
         <v>--</v>
@@ -7445,25 +7445,25 @@
         <v>4</v>
       </c>
       <c r="F100">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G100" t="str">
-        <v>完銷 100%</v>
+        <v>50% (2/4戶)</v>
       </c>
       <c r="H100" t="str">
-        <v>100%</v>
+        <v>50%</v>
       </c>
       <c r="I100">
-        <v>23.9</v>
+        <v>17.7</v>
       </c>
       <c r="J100" t="str">
-        <v>17.1 ~ 30</v>
+        <v>17.1 ~ 18.1</v>
       </c>
       <c r="K100">
-        <v>1019.4</v>
+        <v>1076.7</v>
       </c>
       <c r="L100" t="str">
-        <v>115/01/21</v>
+        <v>111/06/04</v>
       </c>
       <c r="M100" t="str">
         <v>--</v>
@@ -7525,16 +7525,16 @@
         <v>100%</v>
       </c>
       <c r="I101">
-        <v>25.2</v>
+        <v>24.5</v>
       </c>
       <c r="J101" t="str">
-        <v>23.8 ~ 27</v>
+        <v>24 ~ 25.5</v>
       </c>
       <c r="K101">
-        <v>823.1</v>
+        <v>968.3</v>
       </c>
       <c r="L101" t="str">
-        <v>113/04/28</v>
+        <v>112/04/25</v>
       </c>
       <c r="M101">
         <v>16.2</v>
@@ -9007,25 +9007,25 @@
         <v>9</v>
       </c>
       <c r="F122">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G122" t="str">
-        <v>完銷 100%</v>
+        <v>66.7% (6/9戶)</v>
       </c>
       <c r="H122" t="str">
-        <v>100%</v>
+        <v>66.7%</v>
       </c>
       <c r="I122">
-        <v>26.7</v>
+        <v>21</v>
       </c>
       <c r="J122" t="str">
-        <v>19.7 ~ 30.8</v>
+        <v>19.7 ~ 25.3</v>
       </c>
       <c r="K122">
-        <v>912.5</v>
+        <v>999.1</v>
       </c>
       <c r="L122" t="str">
-        <v>115/05/10</v>
+        <v>111/08/08</v>
       </c>
       <c r="M122" t="str">
         <v>--</v>
@@ -9078,25 +9078,25 @@
         <v>30</v>
       </c>
       <c r="F123">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G123" t="str">
-        <v>90% (27/30戶)</v>
+        <v>63.3% (19/30戶)</v>
       </c>
       <c r="H123" t="str">
-        <v>90%</v>
+        <v>63.3%</v>
       </c>
       <c r="I123">
-        <v>21.8</v>
+        <v>21.6</v>
       </c>
       <c r="J123" t="str">
         <v>20.2 ~ 24.9</v>
       </c>
       <c r="K123">
-        <v>1026.9</v>
+        <v>944</v>
       </c>
       <c r="L123" t="str">
-        <v>113/12/05</v>
+        <v>112/06/28</v>
       </c>
       <c r="M123" t="str">
         <v>--</v>
@@ -9291,25 +9291,25 @@
         <v>8</v>
       </c>
       <c r="F126">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G126" t="str">
-        <v>50% (4/8戶)</v>
+        <v>37.5% (3/8戶)</v>
       </c>
       <c r="H126" t="str">
-        <v>50%</v>
+        <v>37.5%</v>
       </c>
       <c r="I126">
-        <v>39.2</v>
+        <v>38.5</v>
       </c>
       <c r="J126" t="str">
-        <v>36.9 ~ 45.4</v>
+        <v>36.9 ~ 42.4</v>
       </c>
       <c r="K126">
-        <v>2635.3</v>
+        <v>2527.3</v>
       </c>
       <c r="L126" t="str">
-        <v>115/03/06</v>
+        <v>114/05/29</v>
       </c>
       <c r="M126" t="str">
         <v>--</v>
@@ -10995,22 +10995,22 @@
         <v>40</v>
       </c>
       <c r="F150">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="G150" t="str">
-        <v>92.5% (37/40戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H150" t="str">
-        <v>92.5%</v>
+        <v>100%</v>
       </c>
       <c r="I150">
-        <v>24.4</v>
+        <v>21.7</v>
       </c>
       <c r="J150" t="str">
-        <v>23.5 ~ 26.7</v>
+        <v>16.7 ~ 26.7</v>
       </c>
       <c r="K150">
-        <v>640.3</v>
+        <v>691.3</v>
       </c>
       <c r="L150" t="str">
         <v>112/10/09</v>
@@ -15255,25 +15255,25 @@
         <v>8</v>
       </c>
       <c r="F210">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G210" t="str">
-        <v>完銷 100%</v>
+        <v>87.5% (7/8戶)</v>
       </c>
       <c r="H210" t="str">
-        <v>100%</v>
+        <v>87.5%</v>
       </c>
       <c r="I210">
-        <v>22.6</v>
+        <v>22.2</v>
       </c>
       <c r="J210" t="str">
-        <v>21.1 ~ 25.5</v>
+        <v>21.1 ~ 24.1</v>
       </c>
       <c r="K210">
-        <v>854.7</v>
+        <v>911.6</v>
       </c>
       <c r="L210" t="str">
-        <v>115/07/25</v>
+        <v>113/03/24</v>
       </c>
       <c r="M210">
         <v>11.8</v>
@@ -15539,22 +15539,22 @@
         <v>46</v>
       </c>
       <c r="F214">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="G214" t="str">
-        <v>91.3% (42/46戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H214" t="str">
-        <v>91.3%</v>
+        <v>100%</v>
       </c>
       <c r="I214">
-        <v>24.1</v>
+        <v>24.4</v>
       </c>
       <c r="J214" t="str">
-        <v>21 ~ 30.2</v>
+        <v>19.8 ~ 30.2</v>
       </c>
       <c r="K214">
-        <v>683.4</v>
+        <v>728.2</v>
       </c>
       <c r="L214" t="str">
         <v>114/04/29</v>
@@ -18308,22 +18308,22 @@
         <v>81</v>
       </c>
       <c r="F253">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G253" t="str">
-        <v>54.3% (44/81戶)</v>
+        <v>56.8% (46/81戶)</v>
       </c>
       <c r="H253" t="str">
-        <v>54.3%</v>
+        <v>56.8%</v>
       </c>
       <c r="I253">
         <v>26.8</v>
       </c>
       <c r="J253" t="str">
-        <v>24.2 ~ 32</v>
+        <v>22.7 ~ 32</v>
       </c>
       <c r="K253">
-        <v>488</v>
+        <v>491.7</v>
       </c>
       <c r="L253" t="str">
         <v>113/06/19</v>
@@ -18663,22 +18663,22 @@
         <v>6</v>
       </c>
       <c r="F258">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G258" t="str">
-        <v>50% (3/6戶)</v>
+        <v>33.3% (2/6戶)</v>
       </c>
       <c r="H258" t="str">
-        <v>50%</v>
+        <v>33.3%</v>
       </c>
       <c r="I258">
-        <v>23.5</v>
+        <v>22.8</v>
       </c>
       <c r="J258" t="str">
-        <v>21.7 ~ 26.9</v>
+        <v>21.7 ~ 25.4</v>
       </c>
       <c r="K258">
-        <v>1266.8</v>
+        <v>1342.6</v>
       </c>
       <c r="L258" t="str">
         <v>113/12/10</v>
@@ -19018,25 +19018,25 @@
         <v>16</v>
       </c>
       <c r="F263">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G263" t="str">
-        <v>完銷 100%</v>
+        <v>87.5% (14/16戶)</v>
       </c>
       <c r="H263" t="str">
-        <v>100%</v>
+        <v>87.5%</v>
       </c>
       <c r="I263">
-        <v>36.5</v>
+        <v>34.6</v>
       </c>
       <c r="J263" t="str">
-        <v>32.5 ~ 47.5</v>
+        <v>32.5 ~ 37.2</v>
       </c>
       <c r="K263">
-        <v>1145.6</v>
+        <v>1201.5</v>
       </c>
       <c r="L263" t="str">
-        <v>115/03/01</v>
+        <v>114/03/25</v>
       </c>
       <c r="M263">
         <v>19.7</v>
@@ -19444,22 +19444,22 @@
         <v>17</v>
       </c>
       <c r="F269">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G269" t="str">
-        <v>88.2% (15/17戶)</v>
+        <v>94.1% (16/17戶)</v>
       </c>
       <c r="H269" t="str">
-        <v>88.2%</v>
+        <v>94.1%</v>
       </c>
       <c r="I269">
-        <v>33.3</v>
+        <v>32.5</v>
       </c>
       <c r="J269" t="str">
-        <v>30.6 ~ 36.3</v>
+        <v>19.2 ~ 36.3</v>
       </c>
       <c r="K269">
-        <v>895.3</v>
+        <v>886.2</v>
       </c>
       <c r="L269" t="str">
         <v>114/05/31</v>
@@ -20722,22 +20722,22 @@
         <v>6</v>
       </c>
       <c r="F287">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G287" t="str">
-        <v>完銷 100%</v>
+        <v>66.7% (4/6戶)</v>
       </c>
       <c r="H287" t="str">
-        <v>100%</v>
+        <v>66.7%</v>
       </c>
       <c r="I287">
-        <v>24.3</v>
+        <v>24.2</v>
       </c>
       <c r="J287" t="str">
-        <v>22 ~ 27.6</v>
+        <v>22 ~ 26.6</v>
       </c>
       <c r="K287">
-        <v>1421.9</v>
+        <v>1329.2</v>
       </c>
       <c r="L287" t="str">
         <v>114/09/20</v>
@@ -21219,22 +21219,22 @@
         <v>9</v>
       </c>
       <c r="F294">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G294" t="str">
-        <v>77.8% (7/9戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H294" t="str">
-        <v>77.8%</v>
+        <v>100%</v>
       </c>
       <c r="I294">
-        <v>19.4</v>
+        <v>18.9</v>
       </c>
       <c r="J294" t="str">
-        <v>18.2 ~ 20.8</v>
+        <v>16.5 ~ 20.8</v>
       </c>
       <c r="K294">
-        <v>1195.7</v>
+        <v>1223.2</v>
       </c>
       <c r="L294" t="str">
         <v>113/04/27</v>
@@ -21503,25 +21503,25 @@
         <v>12</v>
       </c>
       <c r="F298">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G298" t="str">
-        <v>完銷 100%</v>
+        <v>75% (9/12戶)</v>
       </c>
       <c r="H298" t="str">
-        <v>100%</v>
+        <v>75%</v>
       </c>
       <c r="I298">
-        <v>26</v>
+        <v>26.5</v>
       </c>
       <c r="J298" t="str">
-        <v>23.5 ~ 27.2</v>
+        <v>25.7 ~ 27.2</v>
       </c>
       <c r="K298">
-        <v>677.2</v>
+        <v>685.7</v>
       </c>
       <c r="L298" t="str">
-        <v>115/01/20</v>
+        <v>113/08/24</v>
       </c>
       <c r="M298">
         <v>10.8</v>
@@ -23349,22 +23349,22 @@
         <v>11</v>
       </c>
       <c r="F324">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G324" t="str">
-        <v>36.4% (4/11戶)</v>
+        <v>72.7% (8/11戶)</v>
       </c>
       <c r="H324" t="str">
-        <v>36.4%</v>
+        <v>72.7%</v>
       </c>
       <c r="I324">
-        <v>23.3</v>
+        <v>21.6</v>
       </c>
       <c r="J324" t="str">
-        <v>20.2 ~ 28.9</v>
+        <v>16.5 ~ 28.9</v>
       </c>
       <c r="K324">
-        <v>1199</v>
+        <v>1219.9</v>
       </c>
       <c r="L324" t="str">
         <v>113/12/04</v>
@@ -29668,25 +29668,25 @@
         <v>12</v>
       </c>
       <c r="F413">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G413" t="str">
-        <v>50% (6/12戶)</v>
+        <v>25% (3/12戶)</v>
       </c>
       <c r="H413" t="str">
-        <v>50%</v>
+        <v>25%</v>
       </c>
       <c r="I413">
-        <v>23.5</v>
+        <v>22.7</v>
       </c>
       <c r="J413" t="str">
-        <v>21.3 ~ 25.3</v>
+        <v>21.3 ~ 24.5</v>
       </c>
       <c r="K413">
-        <v>911.5</v>
+        <v>679.7</v>
       </c>
       <c r="L413" t="str">
-        <v>114/09/09</v>
+        <v>114/02/07</v>
       </c>
       <c r="M413">
         <v>10.2</v>

</xml_diff>

<commit_message>
Optimize full lifecycle pre-sale + completed sales counting, fix over-deduplication on large apartment complexes, add source badges
</commit_message>
<xml_diff>
--- a/宜蘭建案實價登錄銷售統計.xlsx
+++ b/宜蘭建案實價登錄銷售統計.xlsx
@@ -487,13 +487,13 @@
         <v>33</v>
       </c>
       <c r="F2">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="G2" t="str">
-        <v>33.3% (11/33戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H2" t="str">
-        <v>33.3%</v>
+        <v>100%</v>
       </c>
       <c r="I2">
         <v>19</v>
@@ -700,13 +700,13 @@
         <v>59</v>
       </c>
       <c r="F5">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G5" t="str">
-        <v>88.1% (52/59戶)</v>
+        <v>91.5% (54/59戶)</v>
       </c>
       <c r="H5" t="str">
-        <v>88.1%</v>
+        <v>91.5%</v>
       </c>
       <c r="I5">
         <v>25.5</v>
@@ -771,13 +771,13 @@
         <v>16</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G6" t="str">
-        <v>25% (4/16戶)</v>
+        <v>93.8% (15/16戶)</v>
       </c>
       <c r="H6" t="str">
-        <v>25%</v>
+        <v>93.8%</v>
       </c>
       <c r="I6">
         <v>13.6</v>
@@ -842,13 +842,13 @@
         <v>46</v>
       </c>
       <c r="F7">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G7" t="str">
-        <v>65.2% (30/46戶)</v>
+        <v>69.6% (32/46戶)</v>
       </c>
       <c r="H7" t="str">
-        <v>65.2%</v>
+        <v>69.6%</v>
       </c>
       <c r="I7">
         <v>19.7</v>
@@ -1126,13 +1126,13 @@
         <v>18</v>
       </c>
       <c r="F11">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="G11" t="str">
-        <v>33.3% (6/18戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H11" t="str">
-        <v>33.3%</v>
+        <v>100%</v>
       </c>
       <c r="I11">
         <v>16.4</v>
@@ -1268,13 +1268,13 @@
         <v>24</v>
       </c>
       <c r="F13">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G13" t="str">
-        <v>83.3% (20/24戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H13" t="str">
-        <v>83.3%</v>
+        <v>100%</v>
       </c>
       <c r="I13">
         <v>18.4</v>
@@ -1339,13 +1339,13 @@
         <v>28</v>
       </c>
       <c r="F14">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="G14" t="str">
-        <v>10.7% (3/28戶)</v>
+        <v>85.7% (24/28戶)</v>
       </c>
       <c r="H14" t="str">
-        <v>10.7%</v>
+        <v>85.7%</v>
       </c>
       <c r="I14">
         <v>22.9</v>
@@ -1410,13 +1410,13 @@
         <v>39</v>
       </c>
       <c r="F15">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="G15" t="str">
-        <v>76.9% (30/39戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H15" t="str">
-        <v>76.9%</v>
+        <v>100%</v>
       </c>
       <c r="I15">
         <v>18.8</v>
@@ -1481,13 +1481,13 @@
         <v>18</v>
       </c>
       <c r="F16">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G16" t="str">
-        <v>44.4% (8/18戶)</v>
+        <v>50% (9/18戶)</v>
       </c>
       <c r="H16" t="str">
-        <v>44.4%</v>
+        <v>50%</v>
       </c>
       <c r="I16">
         <v>19.7</v>
@@ -1552,13 +1552,13 @@
         <v>128</v>
       </c>
       <c r="F17">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G17" t="str">
-        <v>27.3% (35/128戶)</v>
+        <v>28.1% (36/128戶)</v>
       </c>
       <c r="H17" t="str">
-        <v>27.3%</v>
+        <v>28.1%</v>
       </c>
       <c r="I17">
         <v>31.3</v>
@@ -1623,13 +1623,13 @@
         <v>45</v>
       </c>
       <c r="F18">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G18" t="str">
-        <v>88.9% (40/45戶)</v>
+        <v>97.8% (44/45戶)</v>
       </c>
       <c r="H18" t="str">
-        <v>88.9%</v>
+        <v>97.8%</v>
       </c>
       <c r="I18">
         <v>21.8</v>
@@ -1694,13 +1694,13 @@
         <v>247</v>
       </c>
       <c r="F19">
-        <v>146</v>
+        <v>247</v>
       </c>
       <c r="G19" t="str">
-        <v>59.1% (146/247戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H19" t="str">
-        <v>59.1%</v>
+        <v>100%</v>
       </c>
       <c r="I19">
         <v>18.6</v>
@@ -1765,13 +1765,13 @@
         <v>4</v>
       </c>
       <c r="F20">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G20" t="str">
-        <v>75% (3/4戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H20" t="str">
-        <v>75%</v>
+        <v>100%</v>
       </c>
       <c r="I20">
         <v>17.9</v>
@@ -1836,13 +1836,13 @@
         <v>25</v>
       </c>
       <c r="F21">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G21" t="str">
-        <v>28% (7/25戶)</v>
+        <v>32% (8/25戶)</v>
       </c>
       <c r="H21" t="str">
-        <v>28%</v>
+        <v>32%</v>
       </c>
       <c r="I21">
         <v>28.1</v>
@@ -1907,13 +1907,13 @@
         <v>17</v>
       </c>
       <c r="F22">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G22" t="str">
-        <v>76.5% (13/17戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H22" t="str">
-        <v>76.5%</v>
+        <v>100%</v>
       </c>
       <c r="I22">
         <v>19</v>
@@ -1978,13 +1978,13 @@
         <v>89</v>
       </c>
       <c r="F23">
-        <v>45</v>
+        <v>89</v>
       </c>
       <c r="G23" t="str">
-        <v>50.6% (45/89戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H23" t="str">
-        <v>50.6%</v>
+        <v>100%</v>
       </c>
       <c r="I23">
         <v>33.5</v>
@@ -2049,13 +2049,13 @@
         <v>21</v>
       </c>
       <c r="F24">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="G24" t="str">
-        <v>66.7% (14/21戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H24" t="str">
-        <v>66.7%</v>
+        <v>100%</v>
       </c>
       <c r="I24">
         <v>24.8</v>
@@ -2120,13 +2120,13 @@
         <v>30</v>
       </c>
       <c r="F25">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G25" t="str">
-        <v>93.3% (28/30戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H25" t="str">
-        <v>93.3%</v>
+        <v>100%</v>
       </c>
       <c r="I25">
         <v>26.3</v>
@@ -2191,13 +2191,13 @@
         <v>28</v>
       </c>
       <c r="F26">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G26" t="str">
-        <v>78.6% (22/28戶)</v>
+        <v>89.3% (25/28戶)</v>
       </c>
       <c r="H26" t="str">
-        <v>78.6%</v>
+        <v>89.3%</v>
       </c>
       <c r="I26">
         <v>20.4</v>
@@ -2262,13 +2262,13 @@
         <v>20</v>
       </c>
       <c r="F27">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G27" t="str">
-        <v>80% (16/20戶)</v>
+        <v>85% (17/20戶)</v>
       </c>
       <c r="H27" t="str">
-        <v>80%</v>
+        <v>85%</v>
       </c>
       <c r="I27">
         <v>25.3</v>
@@ -2404,13 +2404,13 @@
         <v>10</v>
       </c>
       <c r="F29">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G29" t="str">
-        <v>80% (8/10戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H29" t="str">
-        <v>80%</v>
+        <v>100%</v>
       </c>
       <c r="I29">
         <v>22.1</v>
@@ -2546,13 +2546,13 @@
         <v>16</v>
       </c>
       <c r="F31">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="G31" t="str">
-        <v>31.3% (5/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H31" t="str">
-        <v>31.3%</v>
+        <v>100%</v>
       </c>
       <c r="I31">
         <v>19.2</v>
@@ -2617,13 +2617,13 @@
         <v>21</v>
       </c>
       <c r="F32">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G32" t="str">
-        <v>38.1% (8/21戶)</v>
+        <v>95.2% (20/21戶)</v>
       </c>
       <c r="H32" t="str">
-        <v>38.1%</v>
+        <v>95.2%</v>
       </c>
       <c r="I32">
         <v>18.5</v>
@@ -2688,13 +2688,13 @@
         <v>12</v>
       </c>
       <c r="F33">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G33" t="str">
-        <v>50% (6/12戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H33" t="str">
-        <v>50%</v>
+        <v>100%</v>
       </c>
       <c r="I33">
         <v>22.3</v>
@@ -2901,13 +2901,13 @@
         <v>9</v>
       </c>
       <c r="F36">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G36" t="str">
-        <v>77.8% (7/9戶)</v>
+        <v>88.9% (8/9戶)</v>
       </c>
       <c r="H36" t="str">
-        <v>77.8%</v>
+        <v>88.9%</v>
       </c>
       <c r="I36">
         <v>22.7</v>
@@ -3256,13 +3256,13 @@
         <v>13</v>
       </c>
       <c r="F41">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G41" t="str">
-        <v>69.2% (9/13戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H41" t="str">
-        <v>69.2%</v>
+        <v>100%</v>
       </c>
       <c r="I41">
         <v>21</v>
@@ -3327,13 +3327,13 @@
         <v>10</v>
       </c>
       <c r="F42">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G42" t="str">
-        <v>50% (5/10戶)</v>
+        <v>90% (9/10戶)</v>
       </c>
       <c r="H42" t="str">
-        <v>50%</v>
+        <v>90%</v>
       </c>
       <c r="I42">
         <v>22</v>
@@ -3611,13 +3611,13 @@
         <v>51</v>
       </c>
       <c r="F46">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="G46" t="str">
-        <v>49% (25/51戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H46" t="str">
-        <v>49%</v>
+        <v>100%</v>
       </c>
       <c r="I46">
         <v>19.1</v>
@@ -3753,13 +3753,13 @@
         <v>30</v>
       </c>
       <c r="F48">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G48" t="str">
-        <v>86.7% (26/30戶)</v>
+        <v>96.7% (29/30戶)</v>
       </c>
       <c r="H48" t="str">
-        <v>86.7%</v>
+        <v>96.7%</v>
       </c>
       <c r="I48">
         <v>22.7</v>
@@ -3895,13 +3895,13 @@
         <v>16</v>
       </c>
       <c r="F50">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G50" t="str">
-        <v>68.8% (11/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H50" t="str">
-        <v>68.8%</v>
+        <v>100%</v>
       </c>
       <c r="I50">
         <v>25.8</v>
@@ -3966,13 +3966,13 @@
         <v>36</v>
       </c>
       <c r="F51">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G51" t="str">
-        <v>91.7% (33/36戶)</v>
+        <v>97.2% (35/36戶)</v>
       </c>
       <c r="H51" t="str">
-        <v>91.7%</v>
+        <v>97.2%</v>
       </c>
       <c r="I51">
         <v>25.6</v>
@@ -4321,13 +4321,13 @@
         <v>5</v>
       </c>
       <c r="F56">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G56" t="str">
-        <v>40% (2/5戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H56" t="str">
-        <v>40%</v>
+        <v>100%</v>
       </c>
       <c r="I56">
         <v>17.9</v>
@@ -4392,13 +4392,13 @@
         <v>9</v>
       </c>
       <c r="F57">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G57" t="str">
-        <v>55.6% (5/9戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H57" t="str">
-        <v>55.6%</v>
+        <v>100%</v>
       </c>
       <c r="I57">
         <v>29.8</v>
@@ -4463,13 +4463,13 @@
         <v>22</v>
       </c>
       <c r="F58">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="G58" t="str">
-        <v>45.5% (10/22戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H58" t="str">
-        <v>45.5%</v>
+        <v>100%</v>
       </c>
       <c r="I58">
         <v>19.9</v>
@@ -4605,13 +4605,13 @@
         <v>41</v>
       </c>
       <c r="F60">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="G60" t="str">
-        <v>75.6% (31/41戶)</v>
+        <v>87.8% (36/41戶)</v>
       </c>
       <c r="H60" t="str">
-        <v>75.6%</v>
+        <v>87.8%</v>
       </c>
       <c r="I60">
         <v>19.6</v>
@@ -4676,13 +4676,13 @@
         <v>22</v>
       </c>
       <c r="F61">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G61" t="str">
-        <v>86.4% (19/22戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H61" t="str">
-        <v>86.4%</v>
+        <v>100%</v>
       </c>
       <c r="I61">
         <v>16.9</v>
@@ -4747,13 +4747,13 @@
         <v>14</v>
       </c>
       <c r="F62">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G62" t="str">
-        <v>35.7% (5/14戶)</v>
+        <v>78.6% (11/14戶)</v>
       </c>
       <c r="H62" t="str">
-        <v>35.7%</v>
+        <v>78.6%</v>
       </c>
       <c r="I62">
         <v>18.3</v>
@@ -4818,13 +4818,13 @@
         <v>32</v>
       </c>
       <c r="F63">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="G63" t="str">
-        <v>71.9% (23/32戶)</v>
+        <v>93.8% (30/32戶)</v>
       </c>
       <c r="H63" t="str">
-        <v>71.9%</v>
+        <v>93.8%</v>
       </c>
       <c r="I63">
         <v>15.9</v>
@@ -4889,13 +4889,13 @@
         <v>21</v>
       </c>
       <c r="F64">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G64" t="str">
-        <v>81% (17/21戶)</v>
+        <v>95.2% (20/21戶)</v>
       </c>
       <c r="H64" t="str">
-        <v>81%</v>
+        <v>95.2%</v>
       </c>
       <c r="I64">
         <v>19.4</v>
@@ -5173,13 +5173,13 @@
         <v>16</v>
       </c>
       <c r="F68">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="G68" t="str">
-        <v>37.5% (6/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H68" t="str">
-        <v>37.5%</v>
+        <v>100%</v>
       </c>
       <c r="I68">
         <v>20</v>
@@ -5244,13 +5244,13 @@
         <v>18</v>
       </c>
       <c r="F69">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G69" t="str">
-        <v>83.3% (15/18戶)</v>
+        <v>88.9% (16/18戶)</v>
       </c>
       <c r="H69" t="str">
-        <v>83.3%</v>
+        <v>88.9%</v>
       </c>
       <c r="I69">
         <v>20.9</v>
@@ -5315,13 +5315,13 @@
         <v>7</v>
       </c>
       <c r="F70">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G70" t="str">
-        <v>71.4% (5/7戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H70" t="str">
-        <v>71.4%</v>
+        <v>100%</v>
       </c>
       <c r="I70">
         <v>19.9</v>
@@ -5457,13 +5457,13 @@
         <v>36</v>
       </c>
       <c r="F72">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="G72" t="str">
-        <v>61.1% (22/36戶)</v>
+        <v>97.2% (35/36戶)</v>
       </c>
       <c r="H72" t="str">
-        <v>61.1%</v>
+        <v>97.2%</v>
       </c>
       <c r="I72">
         <v>25.2</v>
@@ -5599,13 +5599,13 @@
         <v>32</v>
       </c>
       <c r="F74">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G74" t="str">
-        <v>90.6% (29/32戶)</v>
+        <v>96.9% (31/32戶)</v>
       </c>
       <c r="H74" t="str">
-        <v>90.6%</v>
+        <v>96.9%</v>
       </c>
       <c r="I74">
         <v>26.9</v>
@@ -5670,13 +5670,13 @@
         <v>12</v>
       </c>
       <c r="F75">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G75" t="str">
-        <v>58.3% (7/12戶)</v>
+        <v>91.7% (11/12戶)</v>
       </c>
       <c r="H75" t="str">
-        <v>58.3%</v>
+        <v>91.7%</v>
       </c>
       <c r="I75">
         <v>16.4</v>
@@ -5741,13 +5741,13 @@
         <v>48</v>
       </c>
       <c r="F76">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G76" t="str">
-        <v>87.5% (42/48戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H76" t="str">
-        <v>87.5%</v>
+        <v>100%</v>
       </c>
       <c r="I76">
         <v>23</v>
@@ -5812,13 +5812,13 @@
         <v>14</v>
       </c>
       <c r="F77">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G77" t="str">
-        <v>50% (7/14戶)</v>
+        <v>92.9% (13/14戶)</v>
       </c>
       <c r="H77" t="str">
-        <v>50%</v>
+        <v>92.9%</v>
       </c>
       <c r="I77">
         <v>18.4</v>
@@ -6096,13 +6096,13 @@
         <v>18</v>
       </c>
       <c r="F81">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G81" t="str">
-        <v>55.6% (10/18戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H81" t="str">
-        <v>55.6%</v>
+        <v>100%</v>
       </c>
       <c r="I81">
         <v>26.5</v>
@@ -6167,13 +6167,13 @@
         <v>8</v>
       </c>
       <c r="F82">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G82" t="str">
-        <v>87.5% (7/8戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H82" t="str">
-        <v>87.5%</v>
+        <v>100%</v>
       </c>
       <c r="I82">
         <v>28.7</v>
@@ -6380,13 +6380,13 @@
         <v>20</v>
       </c>
       <c r="F85">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G85" t="str">
-        <v>40% (8/20戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H85" t="str">
-        <v>40%</v>
+        <v>100%</v>
       </c>
       <c r="I85">
         <v>18.1</v>
@@ -6522,13 +6522,13 @@
         <v>40</v>
       </c>
       <c r="F87">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="G87" t="str">
-        <v>42.5% (17/40戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H87" t="str">
-        <v>42.5%</v>
+        <v>100%</v>
       </c>
       <c r="I87">
         <v>18.7</v>
@@ -6593,13 +6593,13 @@
         <v>25</v>
       </c>
       <c r="F88">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G88" t="str">
-        <v>84% (21/25戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H88" t="str">
-        <v>84%</v>
+        <v>100%</v>
       </c>
       <c r="I88">
         <v>19.4</v>
@@ -6664,13 +6664,13 @@
         <v>7</v>
       </c>
       <c r="F89">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G89" t="str">
-        <v>85.7% (6/7戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H89" t="str">
-        <v>85.7%</v>
+        <v>100%</v>
       </c>
       <c r="I89">
         <v>22.7</v>
@@ -6735,13 +6735,13 @@
         <v>72</v>
       </c>
       <c r="F90">
-        <v>38</v>
+        <v>72</v>
       </c>
       <c r="G90" t="str">
-        <v>52.8% (38/72戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H90" t="str">
-        <v>52.8%</v>
+        <v>100%</v>
       </c>
       <c r="I90">
         <v>27.5</v>
@@ -6806,13 +6806,13 @@
         <v>5</v>
       </c>
       <c r="F91">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G91" t="str">
-        <v>60% (3/5戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H91" t="str">
-        <v>60%</v>
+        <v>100%</v>
       </c>
       <c r="I91">
         <v>15.3</v>
@@ -6948,13 +6948,13 @@
         <v>28</v>
       </c>
       <c r="F93">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="G93" t="str">
-        <v>10.7% (3/28戶)</v>
+        <v>96.4% (27/28戶)</v>
       </c>
       <c r="H93" t="str">
-        <v>10.7%</v>
+        <v>96.4%</v>
       </c>
       <c r="I93">
         <v>18.4</v>
@@ -7019,13 +7019,13 @@
         <v>18</v>
       </c>
       <c r="F94">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G94" t="str">
-        <v>77.8% (14/18戶)</v>
+        <v>88.9% (16/18戶)</v>
       </c>
       <c r="H94" t="str">
-        <v>77.8%</v>
+        <v>88.9%</v>
       </c>
       <c r="I94">
         <v>22.9</v>
@@ -7090,13 +7090,13 @@
         <v>11</v>
       </c>
       <c r="F95">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G95" t="str">
-        <v>63.6% (7/11戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H95" t="str">
-        <v>63.6%</v>
+        <v>100%</v>
       </c>
       <c r="I95">
         <v>24.4</v>
@@ -7161,13 +7161,13 @@
         <v>16</v>
       </c>
       <c r="F96">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G96" t="str">
-        <v>93.8% (15/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H96" t="str">
-        <v>93.8%</v>
+        <v>100%</v>
       </c>
       <c r="I96">
         <v>22.6</v>
@@ -7303,13 +7303,13 @@
         <v>7</v>
       </c>
       <c r="F98">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G98" t="str">
-        <v>57.1% (4/7戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H98" t="str">
-        <v>57.1%</v>
+        <v>100%</v>
       </c>
       <c r="I98">
         <v>16.8</v>
@@ -7445,13 +7445,13 @@
         <v>4</v>
       </c>
       <c r="F100">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G100" t="str">
-        <v>50% (2/4戶)</v>
+        <v>75% (3/4戶)</v>
       </c>
       <c r="H100" t="str">
-        <v>50%</v>
+        <v>75%</v>
       </c>
       <c r="I100">
         <v>17.7</v>
@@ -7587,13 +7587,13 @@
         <v>44</v>
       </c>
       <c r="F102">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="G102" t="str">
-        <v>27.3% (12/44戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H102" t="str">
-        <v>27.3%</v>
+        <v>100%</v>
       </c>
       <c r="I102">
         <v>17.3</v>
@@ -7658,13 +7658,13 @@
         <v>12</v>
       </c>
       <c r="F103">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G103" t="str">
-        <v>25% (3/12戶)</v>
+        <v>91.7% (11/12戶)</v>
       </c>
       <c r="H103" t="str">
-        <v>25%</v>
+        <v>91.7%</v>
       </c>
       <c r="I103">
         <v>19.4</v>
@@ -7729,13 +7729,13 @@
         <v>28</v>
       </c>
       <c r="F104">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="G104" t="str">
-        <v>85.7% (24/28戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H104" t="str">
-        <v>85.7%</v>
+        <v>100%</v>
       </c>
       <c r="I104">
         <v>21.4</v>
@@ -7871,13 +7871,13 @@
         <v>16</v>
       </c>
       <c r="F106">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G106" t="str">
-        <v>43.8% (7/16戶)</v>
+        <v>81.3% (13/16戶)</v>
       </c>
       <c r="H106" t="str">
-        <v>43.8%</v>
+        <v>81.3%</v>
       </c>
       <c r="I106">
         <v>18.1</v>
@@ -7942,13 +7942,13 @@
         <v>43</v>
       </c>
       <c r="F107">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G107" t="str">
-        <v>46.5% (20/43戶)</v>
+        <v>69.8% (30/43戶)</v>
       </c>
       <c r="H107" t="str">
-        <v>46.5%</v>
+        <v>69.8%</v>
       </c>
       <c r="I107">
         <v>18.5</v>
@@ -8013,13 +8013,13 @@
         <v>16</v>
       </c>
       <c r="F108">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G108" t="str">
-        <v>81.3% (13/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H108" t="str">
-        <v>81.3%</v>
+        <v>100%</v>
       </c>
       <c r="I108">
         <v>19.5</v>
@@ -8084,13 +8084,13 @@
         <v>12</v>
       </c>
       <c r="F109">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G109" t="str">
-        <v>58.3% (7/12戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H109" t="str">
-        <v>58.3%</v>
+        <v>100%</v>
       </c>
       <c r="I109">
         <v>20</v>
@@ -8297,13 +8297,13 @@
         <v>4</v>
       </c>
       <c r="F112">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G112" t="str">
-        <v>75% (3/4戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H112" t="str">
-        <v>75%</v>
+        <v>100%</v>
       </c>
       <c r="I112">
         <v>23.1</v>
@@ -8368,13 +8368,13 @@
         <v>21</v>
       </c>
       <c r="F113">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="G113" t="str">
-        <v>33.3% (7/21戶)</v>
+        <v>95.2% (20/21戶)</v>
       </c>
       <c r="H113" t="str">
-        <v>33.3%</v>
+        <v>95.2%</v>
       </c>
       <c r="I113">
         <v>17.6</v>
@@ -8510,13 +8510,13 @@
         <v>24</v>
       </c>
       <c r="F115">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G115" t="str">
-        <v>75% (18/24戶)</v>
+        <v>87.5% (21/24戶)</v>
       </c>
       <c r="H115" t="str">
-        <v>75%</v>
+        <v>87.5%</v>
       </c>
       <c r="I115">
         <v>22.2</v>
@@ -8581,13 +8581,13 @@
         <v>21</v>
       </c>
       <c r="F116">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G116" t="str">
-        <v>38.1% (8/21戶)</v>
+        <v>66.7% (14/21戶)</v>
       </c>
       <c r="H116" t="str">
-        <v>38.1%</v>
+        <v>66.7%</v>
       </c>
       <c r="I116">
         <v>46.6</v>
@@ -8652,13 +8652,13 @@
         <v>56</v>
       </c>
       <c r="F117">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="G117" t="str">
-        <v>73.2% (41/56戶)</v>
+        <v>96.4% (54/56戶)</v>
       </c>
       <c r="H117" t="str">
-        <v>73.2%</v>
+        <v>96.4%</v>
       </c>
       <c r="I117">
         <v>32.3</v>
@@ -8794,13 +8794,13 @@
         <v>24</v>
       </c>
       <c r="F119">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="G119" t="str">
-        <v>37.5% (9/24戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H119" t="str">
-        <v>37.5%</v>
+        <v>100%</v>
       </c>
       <c r="I119">
         <v>23.1</v>
@@ -8936,13 +8936,13 @@
         <v>14</v>
       </c>
       <c r="F121">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G121" t="str">
-        <v>64.3% (9/14戶)</v>
+        <v>92.9% (13/14戶)</v>
       </c>
       <c r="H121" t="str">
-        <v>64.3%</v>
+        <v>92.9%</v>
       </c>
       <c r="I121">
         <v>18.9</v>
@@ -9007,13 +9007,13 @@
         <v>9</v>
       </c>
       <c r="F122">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G122" t="str">
-        <v>66.7% (6/9戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H122" t="str">
-        <v>66.7%</v>
+        <v>100%</v>
       </c>
       <c r="I122">
         <v>21</v>
@@ -9078,13 +9078,13 @@
         <v>30</v>
       </c>
       <c r="F123">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="G123" t="str">
-        <v>63.3% (19/30戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H123" t="str">
-        <v>63.3%</v>
+        <v>100%</v>
       </c>
       <c r="I123">
         <v>21.6</v>
@@ -9149,13 +9149,13 @@
         <v>30</v>
       </c>
       <c r="F124">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="G124" t="str">
-        <v>50% (15/30戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H124" t="str">
-        <v>50%</v>
+        <v>100%</v>
       </c>
       <c r="I124">
         <v>18.9</v>
@@ -9220,13 +9220,13 @@
         <v>22</v>
       </c>
       <c r="F125">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G125" t="str">
-        <v>59.1% (13/22戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H125" t="str">
-        <v>59.1%</v>
+        <v>100%</v>
       </c>
       <c r="I125">
         <v>22.9</v>
@@ -9291,13 +9291,13 @@
         <v>8</v>
       </c>
       <c r="F126">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G126" t="str">
-        <v>37.5% (3/8戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H126" t="str">
-        <v>37.5%</v>
+        <v>100%</v>
       </c>
       <c r="I126">
         <v>38.5</v>
@@ -9433,13 +9433,13 @@
         <v>21</v>
       </c>
       <c r="F128">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G128" t="str">
-        <v>19% (4/21戶)</v>
+        <v>71.4% (15/21戶)</v>
       </c>
       <c r="H128" t="str">
-        <v>19%</v>
+        <v>71.4%</v>
       </c>
       <c r="I128">
         <v>27.5</v>
@@ -9504,13 +9504,13 @@
         <v>48</v>
       </c>
       <c r="F129">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="G129" t="str">
-        <v>58.3% (28/48戶)</v>
+        <v>91.7% (44/48戶)</v>
       </c>
       <c r="H129" t="str">
-        <v>58.3%</v>
+        <v>91.7%</v>
       </c>
       <c r="I129">
         <v>21.4</v>
@@ -9575,13 +9575,13 @@
         <v>25</v>
       </c>
       <c r="F130">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="G130" t="str">
-        <v>76% (19/25戶)</v>
+        <v>96% (24/25戶)</v>
       </c>
       <c r="H130" t="str">
-        <v>76%</v>
+        <v>96%</v>
       </c>
       <c r="I130">
         <v>25.7</v>
@@ -9717,13 +9717,13 @@
         <v>31</v>
       </c>
       <c r="F132">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G132" t="str">
-        <v>80.6% (25/31戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H132" t="str">
-        <v>80.6%</v>
+        <v>100%</v>
       </c>
       <c r="I132">
         <v>20.7</v>
@@ -9930,13 +9930,13 @@
         <v>34</v>
       </c>
       <c r="F135">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="G135" t="str">
-        <v>52.9% (18/34戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H135" t="str">
-        <v>52.9%</v>
+        <v>100%</v>
       </c>
       <c r="I135">
         <v>31.8</v>
@@ -10001,13 +10001,13 @@
         <v>31</v>
       </c>
       <c r="F136">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G136" t="str">
-        <v>58.1% (18/31戶)</v>
+        <v>87.1% (27/31戶)</v>
       </c>
       <c r="H136" t="str">
-        <v>58.1%</v>
+        <v>87.1%</v>
       </c>
       <c r="I136">
         <v>36.6</v>
@@ -10072,13 +10072,13 @@
         <v>12</v>
       </c>
       <c r="F137">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G137" t="str">
-        <v>25% (3/12戶)</v>
+        <v>91.7% (11/12戶)</v>
       </c>
       <c r="H137" t="str">
-        <v>25%</v>
+        <v>91.7%</v>
       </c>
       <c r="I137">
         <v>22.4</v>
@@ -10143,13 +10143,13 @@
         <v>23</v>
       </c>
       <c r="F138">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="G138" t="str">
-        <v>47.8% (11/23戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H138" t="str">
-        <v>47.8%</v>
+        <v>100%</v>
       </c>
       <c r="I138">
         <v>18.6</v>
@@ -10285,13 +10285,13 @@
         <v>9</v>
       </c>
       <c r="F140">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G140" t="str">
-        <v>88.9% (8/9戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H140" t="str">
-        <v>88.9%</v>
+        <v>100%</v>
       </c>
       <c r="I140">
         <v>21.6</v>
@@ -10356,13 +10356,13 @@
         <v>25</v>
       </c>
       <c r="F141">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G141" t="str">
-        <v>72% (18/25戶)</v>
+        <v>96% (24/25戶)</v>
       </c>
       <c r="H141" t="str">
-        <v>72%</v>
+        <v>96%</v>
       </c>
       <c r="I141">
         <v>20.5</v>
@@ -10427,13 +10427,13 @@
         <v>32</v>
       </c>
       <c r="F142">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G142" t="str">
-        <v>84.4% (27/32戶)</v>
+        <v>90.6% (29/32戶)</v>
       </c>
       <c r="H142" t="str">
-        <v>84.4%</v>
+        <v>90.6%</v>
       </c>
       <c r="I142">
         <v>25.5</v>
@@ -10498,13 +10498,13 @@
         <v>16</v>
       </c>
       <c r="F143">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G143" t="str">
-        <v>81.3% (13/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H143" t="str">
-        <v>81.3%</v>
+        <v>100%</v>
       </c>
       <c r="I143">
         <v>20.8</v>
@@ -10640,13 +10640,13 @@
         <v>99</v>
       </c>
       <c r="F145">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="G145" t="str">
-        <v>83.8% (83/99戶)</v>
+        <v>96% (95/99戶)</v>
       </c>
       <c r="H145" t="str">
-        <v>83.8%</v>
+        <v>96%</v>
       </c>
       <c r="I145">
         <v>31.8</v>
@@ -10711,13 +10711,13 @@
         <v>22</v>
       </c>
       <c r="F146">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G146" t="str">
-        <v>72.7% (16/22戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H146" t="str">
-        <v>72.7%</v>
+        <v>100%</v>
       </c>
       <c r="I146">
         <v>22.7</v>
@@ -10782,13 +10782,13 @@
         <v>23</v>
       </c>
       <c r="F147">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G147" t="str">
-        <v>87% (20/23戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H147" t="str">
-        <v>87%</v>
+        <v>100%</v>
       </c>
       <c r="I147">
         <v>25.7</v>
@@ -10853,13 +10853,13 @@
         <v>4</v>
       </c>
       <c r="F148">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G148" t="str">
-        <v>75% (3/4戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H148" t="str">
-        <v>75%</v>
+        <v>100%</v>
       </c>
       <c r="I148">
         <v>25.3</v>
@@ -10924,13 +10924,13 @@
         <v>10</v>
       </c>
       <c r="F149">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G149" t="str">
-        <v>30% (3/10戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H149" t="str">
-        <v>30%</v>
+        <v>100%</v>
       </c>
       <c r="I149">
         <v>18.9</v>
@@ -11066,13 +11066,13 @@
         <v>31</v>
       </c>
       <c r="F151">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G151" t="str">
-        <v>74.2% (23/31戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H151" t="str">
-        <v>74.2%</v>
+        <v>100%</v>
       </c>
       <c r="I151">
         <v>22.5</v>
@@ -11208,13 +11208,13 @@
         <v>11</v>
       </c>
       <c r="F153">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G153" t="str">
-        <v>81.8% (9/11戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H153" t="str">
-        <v>81.8%</v>
+        <v>100%</v>
       </c>
       <c r="I153">
         <v>22.7</v>
@@ -11279,13 +11279,13 @@
         <v>44</v>
       </c>
       <c r="F154">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="G154" t="str">
-        <v>81.8% (36/44戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H154" t="str">
-        <v>81.8%</v>
+        <v>100%</v>
       </c>
       <c r="I154">
         <v>17.5</v>
@@ -11421,13 +11421,13 @@
         <v>102</v>
       </c>
       <c r="F156">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="G156" t="str">
-        <v>73.5% (75/102戶)</v>
+        <v>98% (100/102戶)</v>
       </c>
       <c r="H156" t="str">
-        <v>73.5%</v>
+        <v>98%</v>
       </c>
       <c r="I156">
         <v>29</v>
@@ -11634,13 +11634,13 @@
         <v>10</v>
       </c>
       <c r="F159">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G159" t="str">
-        <v>80% (8/10戶)</v>
+        <v>90% (9/10戶)</v>
       </c>
       <c r="H159" t="str">
-        <v>80%</v>
+        <v>90%</v>
       </c>
       <c r="I159">
         <v>29.4</v>
@@ -11776,13 +11776,13 @@
         <v>11</v>
       </c>
       <c r="F161">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G161" t="str">
-        <v>45.5% (5/11戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H161" t="str">
-        <v>45.5%</v>
+        <v>100%</v>
       </c>
       <c r="I161">
         <v>23.3</v>
@@ -11918,13 +11918,13 @@
         <v>10</v>
       </c>
       <c r="F163">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G163" t="str">
-        <v>70% (7/10戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H163" t="str">
-        <v>70%</v>
+        <v>100%</v>
       </c>
       <c r="I163">
         <v>20.6</v>
@@ -11989,13 +11989,13 @@
         <v>16</v>
       </c>
       <c r="F164">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="G164" t="str">
-        <v>43.8% (7/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H164" t="str">
-        <v>43.8%</v>
+        <v>100%</v>
       </c>
       <c r="I164">
         <v>18.3</v>
@@ -12202,13 +12202,13 @@
         <v>47</v>
       </c>
       <c r="F167">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G167" t="str">
-        <v>70.2% (33/47戶)</v>
+        <v>72.3% (34/47戶)</v>
       </c>
       <c r="H167" t="str">
-        <v>70.2%</v>
+        <v>72.3%</v>
       </c>
       <c r="I167">
         <v>37.4</v>
@@ -12273,13 +12273,13 @@
         <v>27</v>
       </c>
       <c r="F168">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G168" t="str">
-        <v>70.4% (19/27戶)</v>
+        <v>77.8% (21/27戶)</v>
       </c>
       <c r="H168" t="str">
-        <v>70.4%</v>
+        <v>77.8%</v>
       </c>
       <c r="I168">
         <v>26.1</v>
@@ -12344,13 +12344,13 @@
         <v>32</v>
       </c>
       <c r="F169">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="G169" t="str">
-        <v>50% (16/32戶)</v>
+        <v>68.8% (22/32戶)</v>
       </c>
       <c r="H169" t="str">
-        <v>50%</v>
+        <v>68.8%</v>
       </c>
       <c r="I169">
         <v>26</v>
@@ -12415,13 +12415,13 @@
         <v>34</v>
       </c>
       <c r="F170">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="G170" t="str">
-        <v>38.2% (13/34戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H170" t="str">
-        <v>38.2%</v>
+        <v>100%</v>
       </c>
       <c r="I170">
         <v>20.3</v>
@@ -12486,13 +12486,13 @@
         <v>18</v>
       </c>
       <c r="F171">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="G171" t="str">
-        <v>33.3% (6/18戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H171" t="str">
-        <v>33.3%</v>
+        <v>100%</v>
       </c>
       <c r="I171">
         <v>21.4</v>
@@ -12628,13 +12628,13 @@
         <v>53</v>
       </c>
       <c r="F173">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="G173" t="str">
-        <v>18.9% (10/53戶)</v>
+        <v>77.4% (41/53戶)</v>
       </c>
       <c r="H173" t="str">
-        <v>18.9%</v>
+        <v>77.4%</v>
       </c>
       <c r="I173">
         <v>23.2</v>
@@ -12699,13 +12699,13 @@
         <v>18</v>
       </c>
       <c r="F174">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="G174" t="str">
-        <v>27.8% (5/18戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H174" t="str">
-        <v>27.8%</v>
+        <v>100%</v>
       </c>
       <c r="I174">
         <v>21.4</v>
@@ -12770,13 +12770,13 @@
         <v>44</v>
       </c>
       <c r="F175">
-        <v>5</v>
+        <v>44</v>
       </c>
       <c r="G175" t="str">
-        <v>11.4% (5/44戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H175" t="str">
-        <v>11.4%</v>
+        <v>100%</v>
       </c>
       <c r="I175">
         <v>24.5</v>
@@ -12983,13 +12983,13 @@
         <v>17</v>
       </c>
       <c r="F178">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G178" t="str">
-        <v>29.4% (5/17戶)</v>
+        <v>70.6% (12/17戶)</v>
       </c>
       <c r="H178" t="str">
-        <v>29.4%</v>
+        <v>70.6%</v>
       </c>
       <c r="I178">
         <v>20.6</v>
@@ -13054,13 +13054,13 @@
         <v>30</v>
       </c>
       <c r="F179">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="G179" t="str">
-        <v>73.3% (22/30戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H179" t="str">
-        <v>73.3%</v>
+        <v>100%</v>
       </c>
       <c r="I179">
         <v>33</v>
@@ -13196,13 +13196,13 @@
         <v>62</v>
       </c>
       <c r="F181">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G181" t="str">
-        <v>83.9% (52/62戶)</v>
+        <v>87.1% (54/62戶)</v>
       </c>
       <c r="H181" t="str">
-        <v>83.9%</v>
+        <v>87.1%</v>
       </c>
       <c r="I181">
         <v>41.2</v>
@@ -13338,13 +13338,13 @@
         <v>43</v>
       </c>
       <c r="F183">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G183" t="str">
-        <v>88.4% (38/43戶)</v>
+        <v>97.7% (42/43戶)</v>
       </c>
       <c r="H183" t="str">
-        <v>88.4%</v>
+        <v>97.7%</v>
       </c>
       <c r="I183">
         <v>27.1</v>
@@ -13551,13 +13551,13 @@
         <v>69</v>
       </c>
       <c r="F186">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="G186" t="str">
-        <v>84.1% (58/69戶)</v>
+        <v>97.1% (67/69戶)</v>
       </c>
       <c r="H186" t="str">
-        <v>84.1%</v>
+        <v>97.1%</v>
       </c>
       <c r="I186">
         <v>24.4</v>
@@ -13622,13 +13622,13 @@
         <v>28</v>
       </c>
       <c r="F187">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G187" t="str">
-        <v>35.7% (10/28戶)</v>
+        <v>82.1% (23/28戶)</v>
       </c>
       <c r="H187" t="str">
-        <v>35.7%</v>
+        <v>82.1%</v>
       </c>
       <c r="I187">
         <v>19.7</v>
@@ -13693,13 +13693,13 @@
         <v>13</v>
       </c>
       <c r="F188">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G188" t="str">
-        <v>15.4% (2/13戶)</v>
+        <v>92.3% (12/13戶)</v>
       </c>
       <c r="H188" t="str">
-        <v>15.4%</v>
+        <v>92.3%</v>
       </c>
       <c r="I188">
         <v>19.6</v>
@@ -14048,13 +14048,13 @@
         <v>29</v>
       </c>
       <c r="F193">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="G193" t="str">
-        <v>17.2% (5/29戶)</v>
+        <v>82.8% (24/29戶)</v>
       </c>
       <c r="H193" t="str">
-        <v>17.2%</v>
+        <v>82.8%</v>
       </c>
       <c r="I193">
         <v>18.9</v>
@@ -14119,13 +14119,13 @@
         <v>43</v>
       </c>
       <c r="F194">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G194" t="str">
-        <v>69.8% (30/43戶)</v>
+        <v>93% (40/43戶)</v>
       </c>
       <c r="H194" t="str">
-        <v>69.8%</v>
+        <v>93%</v>
       </c>
       <c r="I194">
         <v>21.3</v>
@@ -14190,13 +14190,13 @@
         <v>33</v>
       </c>
       <c r="F195">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="G195" t="str">
-        <v>36.4% (12/33戶)</v>
+        <v>93.9% (31/33戶)</v>
       </c>
       <c r="H195" t="str">
-        <v>36.4%</v>
+        <v>93.9%</v>
       </c>
       <c r="I195">
         <v>17.9</v>
@@ -14332,13 +14332,13 @@
         <v>13</v>
       </c>
       <c r="F197">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G197" t="str">
-        <v>69.2% (9/13戶)</v>
+        <v>92.3% (12/13戶)</v>
       </c>
       <c r="H197" t="str">
-        <v>69.2%</v>
+        <v>92.3%</v>
       </c>
       <c r="I197">
         <v>19</v>
@@ -14403,13 +14403,13 @@
         <v>30</v>
       </c>
       <c r="F198">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="G198" t="str">
-        <v>66.7% (20/30戶)</v>
+        <v>96.7% (29/30戶)</v>
       </c>
       <c r="H198" t="str">
-        <v>66.7%</v>
+        <v>96.7%</v>
       </c>
       <c r="I198">
         <v>16.9</v>
@@ -14545,13 +14545,13 @@
         <v>15</v>
       </c>
       <c r="F200">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="G200" t="str">
-        <v>46.7% (7/15戶)</v>
+        <v>80% (12/15戶)</v>
       </c>
       <c r="H200" t="str">
-        <v>46.7%</v>
+        <v>80%</v>
       </c>
       <c r="I200">
         <v>22.2</v>
@@ -14758,13 +14758,13 @@
         <v>10</v>
       </c>
       <c r="F203">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G203" t="str">
-        <v>70% (7/10戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H203" t="str">
-        <v>70%</v>
+        <v>100%</v>
       </c>
       <c r="I203">
         <v>26.8</v>
@@ -14900,13 +14900,13 @@
         <v>15</v>
       </c>
       <c r="F205">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="G205" t="str">
-        <v>53.3% (8/15戶)</v>
+        <v>93.3% (14/15戶)</v>
       </c>
       <c r="H205" t="str">
-        <v>53.3%</v>
+        <v>93.3%</v>
       </c>
       <c r="I205">
         <v>29</v>
@@ -14971,13 +14971,13 @@
         <v>36</v>
       </c>
       <c r="F206">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="G206" t="str">
-        <v>77.8% (28/36戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H206" t="str">
-        <v>77.8%</v>
+        <v>100%</v>
       </c>
       <c r="I206">
         <v>20.6</v>
@@ -15042,13 +15042,13 @@
         <v>12</v>
       </c>
       <c r="F207">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G207" t="str">
-        <v>41.7% (5/12戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H207" t="str">
-        <v>41.7%</v>
+        <v>100%</v>
       </c>
       <c r="I207">
         <v>26.2</v>
@@ -15113,13 +15113,13 @@
         <v>6</v>
       </c>
       <c r="F208">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G208" t="str">
-        <v>66.7% (4/6戶)</v>
+        <v>83.3% (5/6戶)</v>
       </c>
       <c r="H208" t="str">
-        <v>66.7%</v>
+        <v>83.3%</v>
       </c>
       <c r="I208">
         <v>20</v>
@@ -15255,13 +15255,13 @@
         <v>8</v>
       </c>
       <c r="F210">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G210" t="str">
-        <v>87.5% (7/8戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H210" t="str">
-        <v>87.5%</v>
+        <v>100%</v>
       </c>
       <c r="I210">
         <v>22.2</v>
@@ -15681,13 +15681,13 @@
         <v>86</v>
       </c>
       <c r="F216">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="G216" t="str">
-        <v>23.3% (20/86戶)</v>
+        <v>59.3% (51/86戶)</v>
       </c>
       <c r="H216" t="str">
-        <v>23.3%</v>
+        <v>59.3%</v>
       </c>
       <c r="I216">
         <v>31.9</v>
@@ -15752,13 +15752,13 @@
         <v>14</v>
       </c>
       <c r="F217">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="G217" t="str">
-        <v>50% (7/14戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H217" t="str">
-        <v>50%</v>
+        <v>100%</v>
       </c>
       <c r="I217">
         <v>24.8</v>
@@ -15965,13 +15965,13 @@
         <v>51</v>
       </c>
       <c r="F220">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="G220" t="str">
-        <v>13.7% (7/51戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H220" t="str">
-        <v>13.7%</v>
+        <v>100%</v>
       </c>
       <c r="I220">
         <v>17.6</v>
@@ -16178,13 +16178,13 @@
         <v>15</v>
       </c>
       <c r="F223">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G223" t="str">
-        <v>60% (9/15戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H223" t="str">
-        <v>60%</v>
+        <v>100%</v>
       </c>
       <c r="I223">
         <v>21</v>
@@ -16249,13 +16249,13 @@
         <v>24</v>
       </c>
       <c r="F224">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G224" t="str">
-        <v>29.2% (7/24戶)</v>
+        <v>54.2% (13/24戶)</v>
       </c>
       <c r="H224" t="str">
-        <v>29.2%</v>
+        <v>54.2%</v>
       </c>
       <c r="I224">
         <v>20</v>
@@ -16320,13 +16320,13 @@
         <v>17</v>
       </c>
       <c r="F225">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G225" t="str">
-        <v>82.4% (14/17戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H225" t="str">
-        <v>82.4%</v>
+        <v>100%</v>
       </c>
       <c r="I225">
         <v>21.6</v>
@@ -16533,13 +16533,13 @@
         <v>14</v>
       </c>
       <c r="F228">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G228" t="str">
-        <v>71.4% (10/14戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H228" t="str">
-        <v>71.4%</v>
+        <v>100%</v>
       </c>
       <c r="I228">
         <v>29</v>
@@ -16604,13 +16604,13 @@
         <v>16</v>
       </c>
       <c r="F229">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="G229" t="str">
-        <v>25% (4/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H229" t="str">
-        <v>25%</v>
+        <v>100%</v>
       </c>
       <c r="I229">
         <v>25</v>
@@ -16675,13 +16675,13 @@
         <v>16</v>
       </c>
       <c r="F230">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G230" t="str">
-        <v>50% (8/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H230" t="str">
-        <v>50%</v>
+        <v>100%</v>
       </c>
       <c r="I230">
         <v>17.7</v>
@@ -16746,13 +16746,13 @@
         <v>14</v>
       </c>
       <c r="F231">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G231" t="str">
-        <v>92.9% (13/14戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H231" t="str">
-        <v>92.9%</v>
+        <v>100%</v>
       </c>
       <c r="I231">
         <v>21.3</v>
@@ -16888,13 +16888,13 @@
         <v>95</v>
       </c>
       <c r="F233">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="G233" t="str">
-        <v>76.8% (73/95戶)</v>
+        <v>93.7% (89/95戶)</v>
       </c>
       <c r="H233" t="str">
-        <v>76.8%</v>
+        <v>93.7%</v>
       </c>
       <c r="I233">
         <v>21.2</v>
@@ -17243,13 +17243,13 @@
         <v>21</v>
       </c>
       <c r="F238">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G238" t="str">
-        <v>66.7% (14/21戶)</v>
+        <v>76.2% (16/21戶)</v>
       </c>
       <c r="H238" t="str">
-        <v>66.7%</v>
+        <v>76.2%</v>
       </c>
       <c r="I238">
         <v>21.6</v>
@@ -17314,13 +17314,13 @@
         <v>34</v>
       </c>
       <c r="F239">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="G239" t="str">
-        <v>17.6% (6/34戶)</v>
+        <v>91.2% (31/34戶)</v>
       </c>
       <c r="H239" t="str">
-        <v>17.6%</v>
+        <v>91.2%</v>
       </c>
       <c r="I239">
         <v>22.2</v>
@@ -17385,13 +17385,13 @@
         <v>54</v>
       </c>
       <c r="F240">
-        <v>33</v>
+        <v>50</v>
       </c>
       <c r="G240" t="str">
-        <v>61.1% (33/54戶)</v>
+        <v>92.6% (50/54戶)</v>
       </c>
       <c r="H240" t="str">
-        <v>61.1%</v>
+        <v>92.6%</v>
       </c>
       <c r="I240">
         <v>26.6</v>
@@ -17456,13 +17456,13 @@
         <v>28</v>
       </c>
       <c r="F241">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G241" t="str">
-        <v>78.6% (22/28戶)</v>
+        <v>85.7% (24/28戶)</v>
       </c>
       <c r="H241" t="str">
-        <v>78.6%</v>
+        <v>85.7%</v>
       </c>
       <c r="I241">
         <v>21.5</v>
@@ -17527,13 +17527,13 @@
         <v>5</v>
       </c>
       <c r="F242">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G242" t="str">
-        <v>40% (2/5戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H242" t="str">
-        <v>40%</v>
+        <v>100%</v>
       </c>
       <c r="I242">
         <v>18.8</v>
@@ -17598,13 +17598,13 @@
         <v>8</v>
       </c>
       <c r="F243">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G243" t="str">
-        <v>50% (4/8戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H243" t="str">
-        <v>50%</v>
+        <v>100%</v>
       </c>
       <c r="I243">
         <v>28.4</v>
@@ -17669,13 +17669,13 @@
         <v>6</v>
       </c>
       <c r="F244">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G244" t="str">
-        <v>66.7% (4/6戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H244" t="str">
-        <v>66.7%</v>
+        <v>100%</v>
       </c>
       <c r="I244">
         <v>25.8</v>
@@ -17811,13 +17811,13 @@
         <v>11</v>
       </c>
       <c r="F246">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G246" t="str">
-        <v>27.3% (3/11戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H246" t="str">
-        <v>27.3%</v>
+        <v>100%</v>
       </c>
       <c r="I246">
         <v>19.6</v>
@@ -17882,13 +17882,13 @@
         <v>14</v>
       </c>
       <c r="F247">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G247" t="str">
-        <v>57.1% (8/14戶)</v>
+        <v>78.6% (11/14戶)</v>
       </c>
       <c r="H247" t="str">
-        <v>57.1%</v>
+        <v>78.6%</v>
       </c>
       <c r="I247">
         <v>22.5</v>
@@ -18024,13 +18024,13 @@
         <v>13</v>
       </c>
       <c r="F249">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G249" t="str">
-        <v>76.9% (10/13戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H249" t="str">
-        <v>76.9%</v>
+        <v>100%</v>
       </c>
       <c r="I249">
         <v>29.6</v>
@@ -18095,13 +18095,13 @@
         <v>31</v>
       </c>
       <c r="F250">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G250" t="str">
-        <v>29% (9/31戶)</v>
+        <v>58.1% (18/31戶)</v>
       </c>
       <c r="H250" t="str">
-        <v>29%</v>
+        <v>58.1%</v>
       </c>
       <c r="I250">
         <v>25</v>
@@ -18166,13 +18166,13 @@
         <v>55</v>
       </c>
       <c r="F251">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="G251" t="str">
-        <v>60% (33/55戶)</v>
+        <v>81.8% (45/55戶)</v>
       </c>
       <c r="H251" t="str">
-        <v>60%</v>
+        <v>81.8%</v>
       </c>
       <c r="I251">
         <v>21.4</v>
@@ -18237,13 +18237,13 @@
         <v>35</v>
       </c>
       <c r="F252">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="G252" t="str">
-        <v>68.6% (24/35戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H252" t="str">
-        <v>68.6%</v>
+        <v>100%</v>
       </c>
       <c r="I252">
         <v>25</v>
@@ -18308,13 +18308,13 @@
         <v>81</v>
       </c>
       <c r="F253">
-        <v>46</v>
+        <v>81</v>
       </c>
       <c r="G253" t="str">
-        <v>56.8% (46/81戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H253" t="str">
-        <v>56.8%</v>
+        <v>100%</v>
       </c>
       <c r="I253">
         <v>26.8</v>
@@ -18663,13 +18663,13 @@
         <v>6</v>
       </c>
       <c r="F258">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G258" t="str">
-        <v>33.3% (2/6戶)</v>
+        <v>83.3% (5/6戶)</v>
       </c>
       <c r="H258" t="str">
-        <v>33.3%</v>
+        <v>83.3%</v>
       </c>
       <c r="I258">
         <v>22.8</v>
@@ -18734,13 +18734,13 @@
         <v>8</v>
       </c>
       <c r="F259">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G259" t="str">
-        <v>25% (2/8戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H259" t="str">
-        <v>25%</v>
+        <v>100%</v>
       </c>
       <c r="I259">
         <v>26.3</v>
@@ -18805,13 +18805,13 @@
         <v>95</v>
       </c>
       <c r="F260">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="G260" t="str">
-        <v>85.3% (81/95戶)</v>
+        <v>96.8% (92/95戶)</v>
       </c>
       <c r="H260" t="str">
-        <v>85.3%</v>
+        <v>96.8%</v>
       </c>
       <c r="I260">
         <v>40.8</v>
@@ -18876,13 +18876,13 @@
         <v>21</v>
       </c>
       <c r="F261">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G261" t="str">
-        <v>71.4% (15/21戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H261" t="str">
-        <v>71.4%</v>
+        <v>100%</v>
       </c>
       <c r="I261">
         <v>25.5</v>
@@ -18947,13 +18947,13 @@
         <v>24</v>
       </c>
       <c r="F262">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="G262" t="str">
-        <v>29.2% (7/24戶)</v>
+        <v>95.8% (23/24戶)</v>
       </c>
       <c r="H262" t="str">
-        <v>29.2%</v>
+        <v>95.8%</v>
       </c>
       <c r="I262">
         <v>22</v>
@@ -19160,13 +19160,13 @@
         <v>21</v>
       </c>
       <c r="F265">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="G265" t="str">
-        <v>71.4% (15/21戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H265" t="str">
-        <v>71.4%</v>
+        <v>100%</v>
       </c>
       <c r="I265">
         <v>23.3</v>
@@ -19231,13 +19231,13 @@
         <v>97</v>
       </c>
       <c r="F266">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="G266" t="str">
-        <v>59.8% (58/97戶)</v>
+        <v>79.4% (77/97戶)</v>
       </c>
       <c r="H266" t="str">
-        <v>59.8%</v>
+        <v>79.4%</v>
       </c>
       <c r="I266">
         <v>26.7</v>
@@ -19373,13 +19373,13 @@
         <v>16</v>
       </c>
       <c r="F268">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="G268" t="str">
-        <v>18.8% (3/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H268" t="str">
-        <v>18.8%</v>
+        <v>100%</v>
       </c>
       <c r="I268">
         <v>22.8</v>
@@ -19515,13 +19515,13 @@
         <v>14</v>
       </c>
       <c r="F270">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="G270" t="str">
-        <v>35.7% (5/14戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H270" t="str">
-        <v>35.7%</v>
+        <v>100%</v>
       </c>
       <c r="I270">
         <v>25.3</v>
@@ -19586,13 +19586,13 @@
         <v>55</v>
       </c>
       <c r="F271">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="G271" t="str">
-        <v>83.6% (46/55戶)</v>
+        <v>96.4% (53/55戶)</v>
       </c>
       <c r="H271" t="str">
-        <v>83.6%</v>
+        <v>96.4%</v>
       </c>
       <c r="I271">
         <v>29.7</v>
@@ -19657,13 +19657,13 @@
         <v>18</v>
       </c>
       <c r="F272">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G272" t="str">
-        <v>50% (9/18戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H272" t="str">
-        <v>50%</v>
+        <v>100%</v>
       </c>
       <c r="I272">
         <v>26.9</v>
@@ -19941,13 +19941,13 @@
         <v>76</v>
       </c>
       <c r="F276">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="G276" t="str">
-        <v>67.1% (51/76戶)</v>
+        <v>96.1% (73/76戶)</v>
       </c>
       <c r="H276" t="str">
-        <v>67.1%</v>
+        <v>96.1%</v>
       </c>
       <c r="I276">
         <v>24.8</v>
@@ -20012,13 +20012,13 @@
         <v>10</v>
       </c>
       <c r="F277">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G277" t="str">
-        <v>60% (6/10戶)</v>
+        <v>80% (8/10戶)</v>
       </c>
       <c r="H277" t="str">
-        <v>60%</v>
+        <v>80%</v>
       </c>
       <c r="I277">
         <v>23.4</v>
@@ -20083,13 +20083,13 @@
         <v>54</v>
       </c>
       <c r="F278">
-        <v>25</v>
+        <v>54</v>
       </c>
       <c r="G278" t="str">
-        <v>46.3% (25/54戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H278" t="str">
-        <v>46.3%</v>
+        <v>100%</v>
       </c>
       <c r="I278">
         <v>25.5</v>
@@ -20225,13 +20225,13 @@
         <v>24</v>
       </c>
       <c r="F280">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G280" t="str">
-        <v>91.7% (22/24戶)</v>
+        <v>95.8% (23/24戶)</v>
       </c>
       <c r="H280" t="str">
-        <v>91.7%</v>
+        <v>95.8%</v>
       </c>
       <c r="I280">
         <v>23.5</v>
@@ -20296,13 +20296,13 @@
         <v>8</v>
       </c>
       <c r="F281">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G281" t="str">
-        <v>12.5% (1/8戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H281" t="str">
-        <v>12.5%</v>
+        <v>100%</v>
       </c>
       <c r="I281">
         <v>20.4</v>
@@ -20438,13 +20438,13 @@
         <v>16</v>
       </c>
       <c r="F283">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="G283" t="str">
-        <v>68.8% (11/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H283" t="str">
-        <v>68.8%</v>
+        <v>100%</v>
       </c>
       <c r="I283">
         <v>22.9</v>
@@ -20580,13 +20580,13 @@
         <v>252</v>
       </c>
       <c r="F285">
-        <v>86</v>
+        <v>207</v>
       </c>
       <c r="G285" t="str">
-        <v>34.1% (86/252戶)</v>
+        <v>82.1% (207/252戶)</v>
       </c>
       <c r="H285" t="str">
-        <v>34.1%</v>
+        <v>82.1%</v>
       </c>
       <c r="I285">
         <v>21.7</v>
@@ -20722,13 +20722,13 @@
         <v>6</v>
       </c>
       <c r="F287">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G287" t="str">
-        <v>66.7% (4/6戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H287" t="str">
-        <v>66.7%</v>
+        <v>100%</v>
       </c>
       <c r="I287">
         <v>24.2</v>
@@ -20793,13 +20793,13 @@
         <v>76</v>
       </c>
       <c r="F288">
-        <v>28</v>
+        <v>72</v>
       </c>
       <c r="G288" t="str">
-        <v>36.8% (28/76戶)</v>
+        <v>94.7% (72/76戶)</v>
       </c>
       <c r="H288" t="str">
-        <v>36.8%</v>
+        <v>94.7%</v>
       </c>
       <c r="I288">
         <v>27.4</v>
@@ -21077,13 +21077,13 @@
         <v>13</v>
       </c>
       <c r="F292">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G292" t="str">
-        <v>92.3% (12/13戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H292" t="str">
-        <v>92.3%</v>
+        <v>100%</v>
       </c>
       <c r="I292">
         <v>23.6</v>
@@ -21148,13 +21148,13 @@
         <v>17</v>
       </c>
       <c r="F293">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G293" t="str">
-        <v>76.5% (13/17戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H293" t="str">
-        <v>76.5%</v>
+        <v>100%</v>
       </c>
       <c r="I293">
         <v>22.5</v>
@@ -21290,13 +21290,13 @@
         <v>73</v>
       </c>
       <c r="F295">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="G295" t="str">
-        <v>82.2% (60/73戶)</v>
+        <v>90.4% (66/73戶)</v>
       </c>
       <c r="H295" t="str">
-        <v>82.2%</v>
+        <v>90.4%</v>
       </c>
       <c r="I295">
         <v>40.6</v>
@@ -21361,13 +21361,13 @@
         <v>109</v>
       </c>
       <c r="F296">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="G296" t="str">
-        <v>65.1% (71/109戶)</v>
+        <v>74.3% (81/109戶)</v>
       </c>
       <c r="H296" t="str">
-        <v>65.1%</v>
+        <v>74.3%</v>
       </c>
       <c r="I296">
         <v>42.4</v>
@@ -21503,13 +21503,13 @@
         <v>12</v>
       </c>
       <c r="F298">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G298" t="str">
-        <v>75% (9/12戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H298" t="str">
-        <v>75%</v>
+        <v>100%</v>
       </c>
       <c r="I298">
         <v>26.5</v>
@@ -21574,13 +21574,13 @@
         <v>16</v>
       </c>
       <c r="F299">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G299" t="str">
-        <v>87.5% (14/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H299" t="str">
-        <v>87.5%</v>
+        <v>100%</v>
       </c>
       <c r="I299">
         <v>29.6</v>
@@ -21716,13 +21716,13 @@
         <v>5</v>
       </c>
       <c r="F301">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G301" t="str">
-        <v>80% (4/5戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H301" t="str">
-        <v>80%</v>
+        <v>100%</v>
       </c>
       <c r="I301">
         <v>33.2</v>
@@ -21787,13 +21787,13 @@
         <v>42</v>
       </c>
       <c r="F302">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G302" t="str">
-        <v>42.9% (18/42戶)</v>
+        <v>47.6% (20/42戶)</v>
       </c>
       <c r="H302" t="str">
-        <v>42.9%</v>
+        <v>47.6%</v>
       </c>
       <c r="I302">
         <v>27.6</v>
@@ -21858,13 +21858,13 @@
         <v>30</v>
       </c>
       <c r="F303">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G303" t="str">
-        <v>80% (24/30戶)</v>
+        <v>83.3% (25/30戶)</v>
       </c>
       <c r="H303" t="str">
-        <v>80%</v>
+        <v>83.3%</v>
       </c>
       <c r="I303">
         <v>32</v>
@@ -22000,13 +22000,13 @@
         <v>15</v>
       </c>
       <c r="F305">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="G305" t="str">
-        <v>20% (3/15戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H305" t="str">
-        <v>20%</v>
+        <v>100%</v>
       </c>
       <c r="I305">
         <v>20.1</v>
@@ -22142,13 +22142,13 @@
         <v>18</v>
       </c>
       <c r="F307">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="G307" t="str">
-        <v>50% (9/18戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H307" t="str">
-        <v>50%</v>
+        <v>100%</v>
       </c>
       <c r="I307">
         <v>22.8</v>
@@ -22213,13 +22213,13 @@
         <v>7</v>
       </c>
       <c r="F308">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G308" t="str">
-        <v>85.7% (6/7戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H308" t="str">
-        <v>85.7%</v>
+        <v>100%</v>
       </c>
       <c r="I308">
         <v>19.7</v>
@@ -22355,13 +22355,13 @@
         <v>17</v>
       </c>
       <c r="F310">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="G310" t="str">
-        <v>11.8% (2/17戶)</v>
+        <v>94.1% (16/17戶)</v>
       </c>
       <c r="H310" t="str">
-        <v>11.8%</v>
+        <v>94.1%</v>
       </c>
       <c r="I310">
         <v>26.7</v>
@@ -22568,13 +22568,13 @@
         <v>18</v>
       </c>
       <c r="F313">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="G313" t="str">
-        <v>44.4% (8/18戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H313" t="str">
-        <v>44.4%</v>
+        <v>100%</v>
       </c>
       <c r="I313">
         <v>26.6</v>
@@ -22639,13 +22639,13 @@
         <v>72</v>
       </c>
       <c r="F314">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="G314" t="str">
-        <v>43.1% (31/72戶)</v>
+        <v>70.8% (51/72戶)</v>
       </c>
       <c r="H314" t="str">
-        <v>43.1%</v>
+        <v>70.8%</v>
       </c>
       <c r="I314">
         <v>28.9</v>
@@ -22710,13 +22710,13 @@
         <v>20</v>
       </c>
       <c r="F315">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G315" t="str">
-        <v>80% (16/20戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H315" t="str">
-        <v>80%</v>
+        <v>100%</v>
       </c>
       <c r="I315">
         <v>27.1</v>
@@ -22781,13 +22781,13 @@
         <v>13</v>
       </c>
       <c r="F316">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G316" t="str">
-        <v>38.5% (5/13戶)</v>
+        <v>84.6% (11/13戶)</v>
       </c>
       <c r="H316" t="str">
-        <v>38.5%</v>
+        <v>84.6%</v>
       </c>
       <c r="I316">
         <v>34.6</v>
@@ -22852,13 +22852,13 @@
         <v>7</v>
       </c>
       <c r="F317">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G317" t="str">
-        <v>85.7% (6/7戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H317" t="str">
-        <v>85.7%</v>
+        <v>100%</v>
       </c>
       <c r="I317">
         <v>24.3</v>
@@ -22994,13 +22994,13 @@
         <v>30</v>
       </c>
       <c r="F319">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="G319" t="str">
-        <v>26.7% (8/30戶)</v>
+        <v>96.7% (29/30戶)</v>
       </c>
       <c r="H319" t="str">
-        <v>26.7%</v>
+        <v>96.7%</v>
       </c>
       <c r="I319">
         <v>21</v>
@@ -23207,13 +23207,13 @@
         <v>6</v>
       </c>
       <c r="F322">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G322" t="str">
-        <v>33.3% (2/6戶)</v>
+        <v>83.3% (5/6戶)</v>
       </c>
       <c r="H322" t="str">
-        <v>33.3%</v>
+        <v>83.3%</v>
       </c>
       <c r="I322">
         <v>20</v>
@@ -23349,13 +23349,13 @@
         <v>11</v>
       </c>
       <c r="F324">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G324" t="str">
-        <v>72.7% (8/11戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H324" t="str">
-        <v>72.7%</v>
+        <v>100%</v>
       </c>
       <c r="I324">
         <v>21.6</v>
@@ -23420,13 +23420,13 @@
         <v>23</v>
       </c>
       <c r="F325">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="G325" t="str">
-        <v>47.8% (11/23戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H325" t="str">
-        <v>47.8%</v>
+        <v>100%</v>
       </c>
       <c r="I325">
         <v>22.7</v>
@@ -23633,13 +23633,13 @@
         <v>118</v>
       </c>
       <c r="F328">
-        <v>72</v>
+        <v>117</v>
       </c>
       <c r="G328" t="str">
-        <v>61% (72/118戶)</v>
+        <v>99.2% (117/118戶)</v>
       </c>
       <c r="H328" t="str">
-        <v>61%</v>
+        <v>99.2%</v>
       </c>
       <c r="I328">
         <v>32</v>
@@ -23775,13 +23775,13 @@
         <v>11</v>
       </c>
       <c r="F330">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G330" t="str">
-        <v>36.4% (4/11戶)</v>
+        <v>90.9% (10/11戶)</v>
       </c>
       <c r="H330" t="str">
-        <v>36.4%</v>
+        <v>90.9%</v>
       </c>
       <c r="I330">
         <v>23.9</v>
@@ -24059,13 +24059,13 @@
         <v>8</v>
       </c>
       <c r="F334">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G334" t="str">
-        <v>25% (2/8戶)</v>
+        <v>50% (4/8戶)</v>
       </c>
       <c r="H334" t="str">
-        <v>25%</v>
+        <v>50%</v>
       </c>
       <c r="I334">
         <v>22.7</v>
@@ -24272,13 +24272,13 @@
         <v>27</v>
       </c>
       <c r="F337">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="G337" t="str">
-        <v>63% (17/27戶)</v>
+        <v>85.2% (23/27戶)</v>
       </c>
       <c r="H337" t="str">
-        <v>63%</v>
+        <v>85.2%</v>
       </c>
       <c r="I337">
         <v>21.6</v>
@@ -24414,13 +24414,13 @@
         <v>22</v>
       </c>
       <c r="F339">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="G339" t="str">
-        <v>13.6% (3/22戶)</v>
+        <v>59.1% (13/22戶)</v>
       </c>
       <c r="H339" t="str">
-        <v>13.6%</v>
+        <v>59.1%</v>
       </c>
       <c r="I339">
         <v>65.2</v>
@@ -24556,13 +24556,13 @@
         <v>16</v>
       </c>
       <c r="F341">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="G341" t="str">
-        <v>31.3% (5/16戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H341" t="str">
-        <v>31.3%</v>
+        <v>100%</v>
       </c>
       <c r="I341">
         <v>34.1</v>
@@ -24627,13 +24627,13 @@
         <v>27</v>
       </c>
       <c r="F342">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G342" t="str">
-        <v>96.3% (26/27戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H342" t="str">
-        <v>96.3%</v>
+        <v>100%</v>
       </c>
       <c r="I342">
         <v>24.1</v>
@@ -24698,13 +24698,13 @@
         <v>13</v>
       </c>
       <c r="F343">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G343" t="str">
-        <v>61.5% (8/13戶)</v>
+        <v>84.6% (11/13戶)</v>
       </c>
       <c r="H343" t="str">
-        <v>61.5%</v>
+        <v>84.6%</v>
       </c>
       <c r="I343">
         <v>19.9</v>
@@ -24840,13 +24840,13 @@
         <v>24</v>
       </c>
       <c r="F345">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G345" t="str">
-        <v>58.3% (14/24戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H345" t="str">
-        <v>58.3%</v>
+        <v>100%</v>
       </c>
       <c r="I345">
         <v>21.3</v>
@@ -24911,13 +24911,13 @@
         <v>39</v>
       </c>
       <c r="F346">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G346" t="str">
-        <v>69.2% (27/39戶)</v>
+        <v>74.4% (29/39戶)</v>
       </c>
       <c r="H346" t="str">
-        <v>69.2%</v>
+        <v>74.4%</v>
       </c>
       <c r="I346">
         <v>33.4</v>
@@ -24982,13 +24982,13 @@
         <v>12</v>
       </c>
       <c r="F347">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G347" t="str">
-        <v>33.3% (4/12戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H347" t="str">
-        <v>33.3%</v>
+        <v>100%</v>
       </c>
       <c r="I347">
         <v>19.6</v>
@@ -25053,13 +25053,13 @@
         <v>13</v>
       </c>
       <c r="F348">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="G348" t="str">
-        <v>69.2% (9/13戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H348" t="str">
-        <v>69.2%</v>
+        <v>100%</v>
       </c>
       <c r="I348">
         <v>22.4</v>
@@ -25124,13 +25124,13 @@
         <v>9</v>
       </c>
       <c r="F349">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G349" t="str">
-        <v>66.7% (6/9戶)</v>
+        <v>88.9% (8/9戶)</v>
       </c>
       <c r="H349" t="str">
-        <v>66.7%</v>
+        <v>88.9%</v>
       </c>
       <c r="I349">
         <v>19.7</v>
@@ -25337,13 +25337,13 @@
         <v>56</v>
       </c>
       <c r="F352">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="G352" t="str">
-        <v>44.6% (25/56戶)</v>
+        <v>48.2% (27/56戶)</v>
       </c>
       <c r="H352" t="str">
-        <v>44.6%</v>
+        <v>48.2%</v>
       </c>
       <c r="I352">
         <v>22.9</v>
@@ -25408,13 +25408,13 @@
         <v>21</v>
       </c>
       <c r="F353">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G353" t="str">
-        <v>61.9% (13/21戶)</v>
+        <v>66.7% (14/21戶)</v>
       </c>
       <c r="H353" t="str">
-        <v>61.9%</v>
+        <v>66.7%</v>
       </c>
       <c r="I353">
         <v>27.8</v>
@@ -25479,13 +25479,13 @@
         <v>10</v>
       </c>
       <c r="F354">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G354" t="str">
-        <v>30% (3/10戶)</v>
+        <v>50% (5/10戶)</v>
       </c>
       <c r="H354" t="str">
-        <v>30%</v>
+        <v>50%</v>
       </c>
       <c r="I354">
         <v>36.9</v>
@@ -25763,13 +25763,13 @@
         <v>30</v>
       </c>
       <c r="F358">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G358" t="str">
-        <v>40% (12/30戶)</v>
+        <v>43.3% (13/30戶)</v>
       </c>
       <c r="H358" t="str">
-        <v>40%</v>
+        <v>43.3%</v>
       </c>
       <c r="I358">
         <v>27.9</v>
@@ -25834,13 +25834,13 @@
         <v>14</v>
       </c>
       <c r="F359">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G359" t="str">
-        <v>35.7% (5/14戶)</v>
+        <v>78.6% (11/14戶)</v>
       </c>
       <c r="H359" t="str">
-        <v>35.7%</v>
+        <v>78.6%</v>
       </c>
       <c r="I359">
         <v>26.5</v>
@@ -25905,13 +25905,13 @@
         <v>19</v>
       </c>
       <c r="F360">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G360" t="str">
-        <v>31.6% (6/19戶)</v>
+        <v>36.8% (7/19戶)</v>
       </c>
       <c r="H360" t="str">
-        <v>31.6%</v>
+        <v>36.8%</v>
       </c>
       <c r="I360">
         <v>40</v>
@@ -25976,13 +25976,13 @@
         <v>24</v>
       </c>
       <c r="F361">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G361" t="str">
-        <v>83.3% (20/24戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H361" t="str">
-        <v>83.3%</v>
+        <v>100%</v>
       </c>
       <c r="I361">
         <v>26.8</v>
@@ -26260,13 +26260,13 @@
         <v>26</v>
       </c>
       <c r="F365">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="G365" t="str">
-        <v>50% (13/26戶)</v>
+        <v>84.6% (22/26戶)</v>
       </c>
       <c r="H365" t="str">
-        <v>50%</v>
+        <v>84.6%</v>
       </c>
       <c r="I365">
         <v>31.4</v>
@@ -26331,13 +26331,13 @@
         <v>11</v>
       </c>
       <c r="F366">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G366" t="str">
-        <v>45.5% (5/11戶)</v>
+        <v>72.7% (8/11戶)</v>
       </c>
       <c r="H366" t="str">
-        <v>45.5%</v>
+        <v>72.7%</v>
       </c>
       <c r="I366">
         <v>28.2</v>
@@ -26544,13 +26544,13 @@
         <v>24</v>
       </c>
       <c r="F369">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="G369" t="str">
-        <v>16.7% (4/24戶)</v>
+        <v>58.3% (14/24戶)</v>
       </c>
       <c r="H369" t="str">
-        <v>16.7%</v>
+        <v>58.3%</v>
       </c>
       <c r="I369">
         <v>23.6</v>
@@ -26615,13 +26615,13 @@
         <v>26</v>
       </c>
       <c r="F370">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G370" t="str">
-        <v>88.5% (23/26戶)</v>
+        <v>92.3% (24/26戶)</v>
       </c>
       <c r="H370" t="str">
-        <v>88.5%</v>
+        <v>92.3%</v>
       </c>
       <c r="I370">
         <v>25.7</v>
@@ -26686,13 +26686,13 @@
         <v>37</v>
       </c>
       <c r="F371">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G371" t="str">
-        <v>43.2% (16/37戶)</v>
+        <v>45.9% (17/37戶)</v>
       </c>
       <c r="H371" t="str">
-        <v>43.2%</v>
+        <v>45.9%</v>
       </c>
       <c r="I371">
         <v>31.2</v>
@@ -26899,13 +26899,13 @@
         <v>15</v>
       </c>
       <c r="F374">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G374" t="str">
-        <v>86.7% (13/15戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H374" t="str">
-        <v>86.7%</v>
+        <v>100%</v>
       </c>
       <c r="I374">
         <v>30</v>
@@ -27112,13 +27112,13 @@
         <v>16</v>
       </c>
       <c r="F377">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G377" t="str">
-        <v>37.5% (6/16戶)</v>
+        <v>50% (8/16戶)</v>
       </c>
       <c r="H377" t="str">
-        <v>37.5%</v>
+        <v>50%</v>
       </c>
       <c r="I377">
         <v>22</v>
@@ -27325,13 +27325,13 @@
         <v>6</v>
       </c>
       <c r="F380">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G380" t="str">
-        <v>33.3% (2/6戶)</v>
+        <v>83.3% (5/6戶)</v>
       </c>
       <c r="H380" t="str">
-        <v>33.3%</v>
+        <v>83.3%</v>
       </c>
       <c r="I380">
         <v>25.1</v>
@@ -27609,13 +27609,13 @@
         <v>52</v>
       </c>
       <c r="F384">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G384" t="str">
-        <v>73.1% (38/52戶)</v>
+        <v>78.8% (41/52戶)</v>
       </c>
       <c r="H384" t="str">
-        <v>73.1%</v>
+        <v>78.8%</v>
       </c>
       <c r="I384">
         <v>24.5</v>
@@ -27680,13 +27680,13 @@
         <v>15</v>
       </c>
       <c r="F385">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G385" t="str">
-        <v>40% (6/15戶)</v>
+        <v>46.7% (7/15戶)</v>
       </c>
       <c r="H385" t="str">
-        <v>40%</v>
+        <v>46.7%</v>
       </c>
       <c r="I385">
         <v>23</v>
@@ -27751,13 +27751,13 @@
         <v>23</v>
       </c>
       <c r="F386">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G386" t="str">
-        <v>34.8% (8/23戶)</v>
+        <v>47.8% (11/23戶)</v>
       </c>
       <c r="H386" t="str">
-        <v>34.8%</v>
+        <v>47.8%</v>
       </c>
       <c r="I386">
         <v>28</v>
@@ -27964,13 +27964,13 @@
         <v>42</v>
       </c>
       <c r="F389">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="G389" t="str">
-        <v>66.7% (28/42戶)</v>
+        <v>95.2% (40/42戶)</v>
       </c>
       <c r="H389" t="str">
-        <v>66.7%</v>
+        <v>95.2%</v>
       </c>
       <c r="I389">
         <v>40.4</v>
@@ -28106,13 +28106,13 @@
         <v>36</v>
       </c>
       <c r="F391">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="G391" t="str">
-        <v>55.6% (20/36戶)</v>
+        <v>61.1% (22/36戶)</v>
       </c>
       <c r="H391" t="str">
-        <v>55.6%</v>
+        <v>61.1%</v>
       </c>
       <c r="I391">
         <v>23.9</v>
@@ -28177,13 +28177,13 @@
         <v>10</v>
       </c>
       <c r="F392">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G392" t="str">
-        <v>70% (7/10戶)</v>
+        <v>90% (9/10戶)</v>
       </c>
       <c r="H392" t="str">
-        <v>70%</v>
+        <v>90%</v>
       </c>
       <c r="I392">
         <v>33.1</v>
@@ -28461,13 +28461,13 @@
         <v>12</v>
       </c>
       <c r="F396">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G396" t="str">
-        <v>50% (6/12戶)</v>
+        <v>58.3% (7/12戶)</v>
       </c>
       <c r="H396" t="str">
-        <v>50%</v>
+        <v>58.3%</v>
       </c>
       <c r="I396">
         <v>23.7</v>
@@ -28603,13 +28603,13 @@
         <v>20</v>
       </c>
       <c r="F398">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G398" t="str">
-        <v>40% (8/20戶)</v>
+        <v>45% (9/20戶)</v>
       </c>
       <c r="H398" t="str">
-        <v>40%</v>
+        <v>45%</v>
       </c>
       <c r="I398">
         <v>35.3</v>
@@ -28745,13 +28745,13 @@
         <v>6</v>
       </c>
       <c r="F400">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G400" t="str">
-        <v>66.7% (4/6戶)</v>
+        <v>83.3% (5/6戶)</v>
       </c>
       <c r="H400" t="str">
-        <v>66.7%</v>
+        <v>83.3%</v>
       </c>
       <c r="I400">
         <v>42.2</v>
@@ -29029,13 +29029,13 @@
         <v>152</v>
       </c>
       <c r="F404">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="G404" t="str">
-        <v>27.6% (42/152戶)</v>
+        <v>32.9% (50/152戶)</v>
       </c>
       <c r="H404" t="str">
-        <v>27.6%</v>
+        <v>32.9%</v>
       </c>
       <c r="I404">
         <v>34.7</v>
@@ -29100,13 +29100,13 @@
         <v>20</v>
       </c>
       <c r="F405">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G405" t="str">
-        <v>70% (14/20戶)</v>
+        <v>75% (15/20戶)</v>
       </c>
       <c r="H405" t="str">
-        <v>70%</v>
+        <v>75%</v>
       </c>
       <c r="I405">
         <v>42.8</v>
@@ -29171,13 +29171,13 @@
         <v>49</v>
       </c>
       <c r="F406">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="G406" t="str">
-        <v>28.6% (14/49戶)</v>
+        <v>67.3% (33/49戶)</v>
       </c>
       <c r="H406" t="str">
-        <v>28.6%</v>
+        <v>67.3%</v>
       </c>
       <c r="I406">
         <v>21.2</v>
@@ -29384,13 +29384,13 @@
         <v>16</v>
       </c>
       <c r="F409">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G409" t="str">
-        <v>25% (4/16戶)</v>
+        <v>50% (8/16戶)</v>
       </c>
       <c r="H409" t="str">
-        <v>25%</v>
+        <v>50%</v>
       </c>
       <c r="I409">
         <v>30.1</v>
@@ -29526,13 +29526,13 @@
         <v>33</v>
       </c>
       <c r="F411">
-        <v>16</v>
+        <v>31</v>
       </c>
       <c r="G411" t="str">
-        <v>48.5% (16/33戶)</v>
+        <v>93.9% (31/33戶)</v>
       </c>
       <c r="H411" t="str">
-        <v>48.5%</v>
+        <v>93.9%</v>
       </c>
       <c r="I411">
         <v>24</v>
@@ -29597,13 +29597,13 @@
         <v>7</v>
       </c>
       <c r="F412">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G412" t="str">
-        <v>28.6% (2/7戶)</v>
+        <v>42.9% (3/7戶)</v>
       </c>
       <c r="H412" t="str">
-        <v>28.6%</v>
+        <v>42.9%</v>
       </c>
       <c r="I412">
         <v>29.3</v>
@@ -29739,13 +29739,13 @@
         <v>35</v>
       </c>
       <c r="F414">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="G414" t="str">
-        <v>28.6% (10/35戶)</v>
+        <v>91.4% (32/35戶)</v>
       </c>
       <c r="H414" t="str">
-        <v>28.6%</v>
+        <v>91.4%</v>
       </c>
       <c r="I414">
         <v>32.4</v>
@@ -29810,13 +29810,13 @@
         <v>123</v>
       </c>
       <c r="F415">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="G415" t="str">
-        <v>8.1% (10/123戶)</v>
+        <v>22.8% (28/123戶)</v>
       </c>
       <c r="H415" t="str">
-        <v>8.1%</v>
+        <v>22.8%</v>
       </c>
       <c r="I415">
         <v>36.3</v>
@@ -30023,13 +30023,13 @@
         <v>9</v>
       </c>
       <c r="F418">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G418" t="str">
-        <v>55.6% (5/9戶)</v>
+        <v>77.8% (7/9戶)</v>
       </c>
       <c r="H418" t="str">
-        <v>55.6%</v>
+        <v>77.8%</v>
       </c>
       <c r="I418">
         <v>24.4</v>
@@ -30094,13 +30094,13 @@
         <v>87</v>
       </c>
       <c r="F419">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G419" t="str">
-        <v>13.8% (12/87戶)</v>
+        <v>21.8% (19/87戶)</v>
       </c>
       <c r="H419" t="str">
-        <v>13.8%</v>
+        <v>21.8%</v>
       </c>
       <c r="I419">
         <v>34.9</v>
@@ -30307,13 +30307,13 @@
         <v>22</v>
       </c>
       <c r="F422">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="G422" t="str">
-        <v>36.4% (8/22戶)</v>
+        <v>95.5% (21/22戶)</v>
       </c>
       <c r="H422" t="str">
-        <v>36.4%</v>
+        <v>95.5%</v>
       </c>
       <c r="I422">
         <v>22.8</v>
@@ -30378,13 +30378,13 @@
         <v>6</v>
       </c>
       <c r="F423">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G423" t="str">
-        <v>16.7% (1/6戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H423" t="str">
-        <v>16.7%</v>
+        <v>100%</v>
       </c>
       <c r="I423">
         <v>29.6</v>
@@ -30662,13 +30662,13 @@
         <v>62</v>
       </c>
       <c r="F427">
-        <v>41</v>
+        <v>62</v>
       </c>
       <c r="G427" t="str">
-        <v>66.1% (41/62戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H427" t="str">
-        <v>66.1%</v>
+        <v>100%</v>
       </c>
       <c r="I427">
         <v>26.4</v>
@@ -31017,13 +31017,13 @@
         <v>37</v>
       </c>
       <c r="F432">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="G432" t="str">
-        <v>24.3% (9/37戶)</v>
+        <v>56.8% (21/37戶)</v>
       </c>
       <c r="H432" t="str">
-        <v>24.3%</v>
+        <v>56.8%</v>
       </c>
       <c r="I432">
         <v>25.6</v>
@@ -31230,13 +31230,13 @@
         <v>37</v>
       </c>
       <c r="F435">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G435" t="str">
-        <v>35.1% (13/37戶)</v>
+        <v>43.2% (16/37戶)</v>
       </c>
       <c r="H435" t="str">
-        <v>35.1%</v>
+        <v>43.2%</v>
       </c>
       <c r="I435">
         <v>32.4</v>
@@ -31301,13 +31301,13 @@
         <v>50</v>
       </c>
       <c r="F436">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="G436" t="str">
-        <v>50% (25/50戶)</v>
+        <v>66% (33/50戶)</v>
       </c>
       <c r="H436" t="str">
-        <v>50%</v>
+        <v>66%</v>
       </c>
       <c r="I436">
         <v>28.3</v>
@@ -31514,13 +31514,13 @@
         <v>15</v>
       </c>
       <c r="F439">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="G439" t="str">
-        <v>40% (6/15戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H439" t="str">
-        <v>40%</v>
+        <v>100%</v>
       </c>
       <c r="I439">
         <v>22</v>
@@ -31798,13 +31798,13 @@
         <v>10</v>
       </c>
       <c r="F443">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G443" t="str">
-        <v>60% (6/10戶)</v>
+        <v>70% (7/10戶)</v>
       </c>
       <c r="H443" t="str">
-        <v>60%</v>
+        <v>70%</v>
       </c>
       <c r="I443">
         <v>25</v>
@@ -31940,13 +31940,13 @@
         <v>8</v>
       </c>
       <c r="F445">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G445" t="str">
-        <v>62.5% (5/8戶)</v>
+        <v>87.5% (7/8戶)</v>
       </c>
       <c r="H445" t="str">
-        <v>62.5%</v>
+        <v>87.5%</v>
       </c>
       <c r="I445">
         <v>21.1</v>
@@ -32011,13 +32011,13 @@
         <v>13</v>
       </c>
       <c r="F446">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G446" t="str">
-        <v>53.8% (7/13戶)</v>
+        <v>61.5% (8/13戶)</v>
       </c>
       <c r="H446" t="str">
-        <v>53.8%</v>
+        <v>61.5%</v>
       </c>
       <c r="I446">
         <v>39.9</v>
@@ -32295,13 +32295,13 @@
         <v>7</v>
       </c>
       <c r="F450">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G450" t="str">
-        <v>14.3% (1/7戶)</v>
+        <v>57.1% (4/7戶)</v>
       </c>
       <c r="H450" t="str">
-        <v>14.3%</v>
+        <v>57.1%</v>
       </c>
       <c r="I450">
         <v>27.1</v>
@@ -32508,13 +32508,13 @@
         <v>30</v>
       </c>
       <c r="F453">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="G453" t="str">
-        <v>26.7% (8/30戶)</v>
+        <v>36.7% (11/30戶)</v>
       </c>
       <c r="H453" t="str">
-        <v>26.7%</v>
+        <v>36.7%</v>
       </c>
       <c r="I453">
         <v>26.3</v>
@@ -32650,13 +32650,13 @@
         <v>15</v>
       </c>
       <c r="F455">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G455" t="str">
-        <v>73.3% (11/15戶)</v>
+        <v>80% (12/15戶)</v>
       </c>
       <c r="H455" t="str">
-        <v>73.3%</v>
+        <v>80%</v>
       </c>
       <c r="I455">
         <v>26</v>
@@ -33715,13 +33715,13 @@
         <v>23</v>
       </c>
       <c r="F470">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="G470" t="str">
-        <v>43.5% (10/23戶)</v>
+        <v>82.6% (19/23戶)</v>
       </c>
       <c r="H470" t="str">
-        <v>43.5%</v>
+        <v>82.6%</v>
       </c>
       <c r="I470">
         <v>23.2</v>
@@ -33786,13 +33786,13 @@
         <v>109</v>
       </c>
       <c r="F471">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="G471" t="str">
-        <v>63.3% (69/109戶)</v>
+        <v>78.9% (86/109戶)</v>
       </c>
       <c r="H471" t="str">
-        <v>63.3%</v>
+        <v>78.9%</v>
       </c>
       <c r="I471">
         <v>42.2</v>
@@ -33857,13 +33857,13 @@
         <v>15</v>
       </c>
       <c r="F472">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G472" t="str">
-        <v>6.7% (1/15戶)</v>
+        <v>26.7% (4/15戶)</v>
       </c>
       <c r="H472" t="str">
-        <v>6.7%</v>
+        <v>26.7%</v>
       </c>
       <c r="I472">
         <v>24.4</v>
@@ -33928,13 +33928,13 @@
         <v>13</v>
       </c>
       <c r="F473">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G473" t="str">
-        <v>15.4% (2/13戶)</v>
+        <v>53.8% (7/13戶)</v>
       </c>
       <c r="H473" t="str">
-        <v>15.4%</v>
+        <v>53.8%</v>
       </c>
       <c r="I473">
         <v>25.5</v>
@@ -33999,13 +33999,13 @@
         <v>11</v>
       </c>
       <c r="F474">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G474" t="str">
-        <v>54.5% (6/11戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H474" t="str">
-        <v>54.5%</v>
+        <v>100%</v>
       </c>
       <c r="I474">
         <v>25</v>
@@ -34070,13 +34070,13 @@
         <v>7</v>
       </c>
       <c r="F475">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G475" t="str">
-        <v>28.6% (2/7戶)</v>
+        <v>57.1% (4/7戶)</v>
       </c>
       <c r="H475" t="str">
-        <v>28.6%</v>
+        <v>57.1%</v>
       </c>
       <c r="I475">
         <v>22.6</v>
@@ -34141,13 +34141,13 @@
         <v>32</v>
       </c>
       <c r="F476">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G476" t="str">
-        <v>3.1% (1/32戶)</v>
+        <v>6.3% (2/32戶)</v>
       </c>
       <c r="H476" t="str">
-        <v>3.1%</v>
+        <v>6.3%</v>
       </c>
       <c r="I476">
         <v>28.9</v>
@@ -34212,13 +34212,13 @@
         <v>7</v>
       </c>
       <c r="F477">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G477" t="str">
-        <v>28.6% (2/7戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H477" t="str">
-        <v>28.6%</v>
+        <v>100%</v>
       </c>
       <c r="I477">
         <v>25.5</v>
@@ -34283,13 +34283,13 @@
         <v>18</v>
       </c>
       <c r="F478">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G478" t="str">
-        <v>16.7% (3/18戶)</v>
+        <v>27.8% (5/18戶)</v>
       </c>
       <c r="H478" t="str">
-        <v>16.7%</v>
+        <v>27.8%</v>
       </c>
       <c r="I478">
         <v>23.8</v>
@@ -34354,13 +34354,13 @@
         <v>8</v>
       </c>
       <c r="F479">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="G479" t="str">
-        <v>25% (2/8戶)</v>
+        <v>完銷 100%</v>
       </c>
       <c r="H479" t="str">
-        <v>25%</v>
+        <v>100%</v>
       </c>
       <c r="I479">
         <v>23.1</v>
@@ -34425,13 +34425,13 @@
         <v>36</v>
       </c>
       <c r="F480">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G480" t="str">
-        <v>27.8% (10/36戶)</v>
+        <v>30.6% (11/36戶)</v>
       </c>
       <c r="H480" t="str">
-        <v>27.8%</v>
+        <v>30.6%</v>
       </c>
       <c r="I480">
         <v>29.1</v>
@@ -34922,13 +34922,13 @@
         <v>14</v>
       </c>
       <c r="F487">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G487" t="str">
-        <v>14.3% (2/14戶)</v>
+        <v>28.6% (4/14戶)</v>
       </c>
       <c r="H487" t="str">
-        <v>14.3%</v>
+        <v>28.6%</v>
       </c>
       <c r="I487">
         <v>28.7</v>
@@ -35064,13 +35064,13 @@
         <v>36</v>
       </c>
       <c r="F489">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G489" t="str">
-        <v>72.2% (26/36戶)</v>
+        <v>86.1% (31/36戶)</v>
       </c>
       <c r="H489" t="str">
-        <v>72.2%</v>
+        <v>86.1%</v>
       </c>
       <c r="I489">
         <v>28.3</v>
@@ -35135,13 +35135,13 @@
         <v>41</v>
       </c>
       <c r="F490">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G490" t="str">
-        <v>34.1% (14/41戶)</v>
+        <v>36.6% (15/41戶)</v>
       </c>
       <c r="H490" t="str">
-        <v>34.1%</v>
+        <v>36.6%</v>
       </c>
       <c r="I490">
         <v>28.6</v>
@@ -35632,13 +35632,13 @@
         <v>30</v>
       </c>
       <c r="F497">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G497" t="str">
-        <v>23.3% (7/30戶)</v>
+        <v>26.7% (8/30戶)</v>
       </c>
       <c r="H497" t="str">
-        <v>23.3%</v>
+        <v>26.7%</v>
       </c>
       <c r="I497">
         <v>24.5</v>
@@ -35703,13 +35703,13 @@
         <v>8</v>
       </c>
       <c r="F498">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G498" t="str">
-        <v>37.5% (3/8戶)</v>
+        <v>87.5% (7/8戶)</v>
       </c>
       <c r="H498" t="str">
-        <v>37.5%</v>
+        <v>87.5%</v>
       </c>
       <c r="I498">
         <v>23.3</v>
@@ -35774,13 +35774,13 @@
         <v>65</v>
       </c>
       <c r="F499">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="G499" t="str">
-        <v>66.2% (43/65戶)</v>
+        <v>87.7% (57/65戶)</v>
       </c>
       <c r="H499" t="str">
-        <v>66.2%</v>
+        <v>87.7%</v>
       </c>
       <c r="I499">
         <v>26.8</v>
@@ -35845,13 +35845,13 @@
         <v>17</v>
       </c>
       <c r="F500">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="G500" t="str">
-        <v>41.2% (7/17戶)</v>
+        <v>82.4% (14/17戶)</v>
       </c>
       <c r="H500" t="str">
-        <v>41.2%</v>
+        <v>82.4%</v>
       </c>
       <c r="I500">
         <v>26.9</v>
@@ -35987,13 +35987,13 @@
         <v>24</v>
       </c>
       <c r="F502">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G502" t="str">
-        <v>33.3% (8/24戶)</v>
+        <v>41.7% (10/24戶)</v>
       </c>
       <c r="H502" t="str">
-        <v>33.3%</v>
+        <v>41.7%</v>
       </c>
       <c r="I502">
         <v>38.5</v>
@@ -36271,13 +36271,13 @@
         <v>40</v>
       </c>
       <c r="F506">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="G506" t="str">
-        <v>15% (6/40戶)</v>
+        <v>75% (30/40戶)</v>
       </c>
       <c r="H506" t="str">
-        <v>15%</v>
+        <v>75%</v>
       </c>
       <c r="I506">
         <v>22.7</v>
@@ -36626,13 +36626,13 @@
         <v>53</v>
       </c>
       <c r="F511">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="G511" t="str">
-        <v>50.9% (27/53戶)</v>
+        <v>73.6% (39/53戶)</v>
       </c>
       <c r="H511" t="str">
-        <v>50.9%</v>
+        <v>73.6%</v>
       </c>
       <c r="I511">
         <v>25.5</v>
@@ -36697,13 +36697,13 @@
         <v>24</v>
       </c>
       <c r="F512">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G512" t="str">
-        <v>20.8% (5/24戶)</v>
+        <v>25% (6/24戶)</v>
       </c>
       <c r="H512" t="str">
-        <v>20.8%</v>
+        <v>25%</v>
       </c>
       <c r="I512">
         <v>20.8</v>
@@ -36839,13 +36839,13 @@
         <v>16</v>
       </c>
       <c r="F514">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G514" t="str">
-        <v>37.5% (6/16戶)</v>
+        <v>50% (8/16戶)</v>
       </c>
       <c r="H514" t="str">
-        <v>37.5%</v>
+        <v>50%</v>
       </c>
       <c r="I514">
         <v>35.2</v>
@@ -37265,13 +37265,13 @@
         <v>12</v>
       </c>
       <c r="F520">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G520" t="str">
-        <v>8.3% (1/12戶)</v>
+        <v>16.7% (2/12戶)</v>
       </c>
       <c r="H520" t="str">
-        <v>8.3%</v>
+        <v>16.7%</v>
       </c>
       <c r="I520">
         <v>41.9</v>
@@ -37904,13 +37904,13 @@
         <v>25</v>
       </c>
       <c r="F529">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G529" t="str">
-        <v>20% (5/25戶)</v>
+        <v>24% (6/25戶)</v>
       </c>
       <c r="H529" t="str">
-        <v>20%</v>
+        <v>24%</v>
       </c>
       <c r="I529">
         <v>22.9</v>
@@ -38188,13 +38188,13 @@
         <v>4</v>
       </c>
       <c r="F533">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G533" t="str">
-        <v>25% (1/4戶)</v>
+        <v>50% (2/4戶)</v>
       </c>
       <c r="H533" t="str">
-        <v>25%</v>
+        <v>50%</v>
       </c>
       <c r="I533">
         <v>26.7</v>
@@ -38898,13 +38898,13 @@
         <v>13</v>
       </c>
       <c r="F543">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G543" t="str">
-        <v>69.2% (9/13戶)</v>
+        <v>76.9% (10/13戶)</v>
       </c>
       <c r="H543" t="str">
-        <v>69.2%</v>
+        <v>76.9%</v>
       </c>
       <c r="I543">
         <v>31</v>
@@ -40105,13 +40105,13 @@
         <v>31</v>
       </c>
       <c r="F560">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G560" t="str">
-        <v>3.2% (1/31戶)</v>
+        <v>6.5% (2/31戶)</v>
       </c>
       <c r="H560" t="str">
-        <v>3.2%</v>
+        <v>6.5%</v>
       </c>
       <c r="I560">
         <v>23.9</v>
@@ -40957,13 +40957,13 @@
         <v>13</v>
       </c>
       <c r="F572">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G572" t="str">
-        <v>7.7% (1/13戶)</v>
+        <v>15.4% (2/13戶)</v>
       </c>
       <c r="H572" t="str">
-        <v>7.7%</v>
+        <v>15.4%</v>
       </c>
       <c r="I572">
         <v>24.3</v>

</xml_diff>

<commit_message>
Update: Refresh local data.json, index.html and Excel stats with 9/21 transactions
</commit_message>
<xml_diff>
--- a/宜蘭建案實價登錄銷售統計.xlsx
+++ b/宜蘭建案實價登錄銷售統計.xlsx
@@ -13736,16 +13736,16 @@
         <v>62</v>
       </c>
       <c r="F181">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G181">
         <v>0</v>
       </c>
       <c r="H181" t="str">
-        <v>87.1% (54/62戶)</v>
+        <v>85.5% (53/62戶)</v>
       </c>
       <c r="I181" t="str">
-        <v>87.1%</v>
+        <v>85.5%</v>
       </c>
       <c r="J181">
         <v>41.2</v>
@@ -13754,10 +13754,10 @@
         <v>35.7 ~ 51.5</v>
       </c>
       <c r="L181">
-        <v>1798.4</v>
+        <v>1799.1</v>
       </c>
       <c r="M181" t="str">
-        <v>115/07/24</v>
+        <v>115/02/09</v>
       </c>
       <c r="N181" t="str">
         <v>--</v>
@@ -21432,16 +21432,16 @@
         <v>252</v>
       </c>
       <c r="F285">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="G285">
         <v>2</v>
       </c>
       <c r="H285" t="str">
-        <v>81.3% (205/252戶)</v>
+        <v>80.6% (203/252戶)</v>
       </c>
       <c r="I285" t="str">
-        <v>81.3%</v>
+        <v>80.6%</v>
       </c>
       <c r="J285">
         <v>21.7</v>
@@ -21450,10 +21450,10 @@
         <v>19.1 ~ 25.4</v>
       </c>
       <c r="L285">
-        <v>522.1</v>
+        <v>522</v>
       </c>
       <c r="M285" t="str">
-        <v>115/07/29</v>
+        <v>115/05/06</v>
       </c>
       <c r="N285" t="str">
         <v>--</v>
@@ -28388,28 +28388,28 @@
         <v>36</v>
       </c>
       <c r="F379">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G379">
         <v>0</v>
       </c>
       <c r="H379" t="str">
-        <v>77.8% (28/36戶)</v>
+        <v>75% (27/36戶)</v>
       </c>
       <c r="I379" t="str">
-        <v>77.8%</v>
+        <v>75%</v>
       </c>
       <c r="J379">
-        <v>31.8</v>
+        <v>31.7</v>
       </c>
       <c r="K379" t="str">
         <v>30 ~ 32.9</v>
       </c>
       <c r="L379">
-        <v>1066.3</v>
+        <v>1060.3</v>
       </c>
       <c r="M379" t="str">
-        <v>115/07/24</v>
+        <v>114/04/01</v>
       </c>
       <c r="N379">
         <v>16.8</v>
@@ -28758,28 +28758,28 @@
         <v>52</v>
       </c>
       <c r="F384">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G384">
         <v>0</v>
       </c>
       <c r="H384" t="str">
-        <v>78.8% (41/52戶)</v>
+        <v>76.9% (40/52戶)</v>
       </c>
       <c r="I384" t="str">
-        <v>78.8%</v>
+        <v>76.9%</v>
       </c>
       <c r="J384">
-        <v>24.5</v>
+        <v>24.4</v>
       </c>
       <c r="K384" t="str">
         <v>22.3 ~ 25.6</v>
       </c>
       <c r="L384">
-        <v>768.9</v>
+        <v>765.9</v>
       </c>
       <c r="M384" t="str">
-        <v>115/07/26</v>
+        <v>115/04/21</v>
       </c>
       <c r="N384">
         <v>6.5</v>
@@ -30238,16 +30238,16 @@
         <v>152</v>
       </c>
       <c r="F404">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G404">
         <v>0</v>
       </c>
       <c r="H404" t="str">
-        <v>32.9% (50/152戶)</v>
+        <v>32.2% (49/152戶)</v>
       </c>
       <c r="I404" t="str">
-        <v>32.9%</v>
+        <v>32.2%</v>
       </c>
       <c r="J404">
         <v>34.7</v>
@@ -30256,10 +30256,10 @@
         <v>28 ~ 43.2</v>
       </c>
       <c r="L404">
-        <v>739</v>
+        <v>737.1</v>
       </c>
       <c r="M404" t="str">
-        <v>115/07/24</v>
+        <v>115/05/06</v>
       </c>
       <c r="N404" t="str">
         <v>--</v>
@@ -30312,28 +30312,28 @@
         <v>20</v>
       </c>
       <c r="F405">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G405">
         <v>0</v>
       </c>
       <c r="H405" t="str">
-        <v>75% (15/20戶)</v>
+        <v>70% (14/20戶)</v>
       </c>
       <c r="I405" t="str">
-        <v>75%</v>
+        <v>70%</v>
       </c>
       <c r="J405">
-        <v>42.8</v>
+        <v>43.2</v>
       </c>
       <c r="K405" t="str">
         <v>36.7 ~ 66.5</v>
       </c>
       <c r="L405">
-        <v>1176</v>
+        <v>1190.7</v>
       </c>
       <c r="M405" t="str">
-        <v>115/07/27</v>
+        <v>115/03/26</v>
       </c>
       <c r="N405">
         <v>33.8</v>
@@ -30756,28 +30756,28 @@
         <v>33</v>
       </c>
       <c r="F411">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G411">
         <v>0</v>
       </c>
       <c r="H411" t="str">
-        <v>93.9% (31/33戶)</v>
+        <v>90.9% (30/33戶)</v>
       </c>
       <c r="I411" t="str">
-        <v>93.9%</v>
+        <v>90.9%</v>
       </c>
       <c r="J411">
-        <v>24</v>
+        <v>23.9</v>
       </c>
       <c r="K411" t="str">
         <v>21 ~ 26.1</v>
       </c>
       <c r="L411">
-        <v>665.8</v>
+        <v>666.5</v>
       </c>
       <c r="M411" t="str">
-        <v>115/07/21</v>
+        <v>115/02/23</v>
       </c>
       <c r="N411">
         <v>10.4</v>
@@ -32754,28 +32754,28 @@
         <v>18</v>
       </c>
       <c r="F438">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G438">
         <v>0</v>
       </c>
       <c r="H438" t="str">
-        <v>尚無實登</v>
+        <v>22.2% (4/18戶)</v>
       </c>
       <c r="I438" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J438" t="str">
-        <v>--</v>
+        <v>22.2%</v>
+      </c>
+      <c r="J438">
+        <v>22.6</v>
       </c>
       <c r="K438" t="str">
-        <v>--</v>
-      </c>
-      <c r="L438" t="str">
-        <v>--</v>
+        <v>22 ~ 23</v>
+      </c>
+      <c r="L438">
+        <v>967.5</v>
       </c>
       <c r="M438" t="str">
-        <v>--</v>
+        <v>115/08/09</v>
       </c>
       <c r="N438" t="str">
         <v>--</v>
@@ -34678,28 +34678,28 @@
         <v>16</v>
       </c>
       <c r="F464">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G464">
         <v>0</v>
       </c>
       <c r="H464" t="str">
-        <v>93.8% (15/16戶)</v>
+        <v>87.5% (14/16戶)</v>
       </c>
       <c r="I464" t="str">
-        <v>93.8%</v>
+        <v>87.5%</v>
       </c>
       <c r="J464">
-        <v>28.7</v>
+        <v>28.8</v>
       </c>
       <c r="K464" t="str">
         <v>27 ~ 30.2</v>
       </c>
       <c r="L464">
-        <v>1017.8</v>
+        <v>1019.1</v>
       </c>
       <c r="M464" t="str">
-        <v>115/07/22</v>
+        <v>115/05/01</v>
       </c>
       <c r="N464">
         <v>10.5</v>
@@ -35196,16 +35196,16 @@
         <v>109</v>
       </c>
       <c r="F471">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="G471">
         <v>0</v>
       </c>
       <c r="H471" t="str">
-        <v>78.9% (86/109戶)</v>
+        <v>79.8% (87/109戶)</v>
       </c>
       <c r="I471" t="str">
-        <v>78.9%</v>
+        <v>79.8%</v>
       </c>
       <c r="J471">
         <v>42.2</v>
@@ -35214,10 +35214,10 @@
         <v>36.9 ~ 51.3</v>
       </c>
       <c r="L471">
-        <v>1552.7</v>
+        <v>1556</v>
       </c>
       <c r="M471" t="str">
-        <v>115/07/30</v>
+        <v>115/08/10</v>
       </c>
       <c r="N471">
         <v>15</v>
@@ -35270,16 +35270,16 @@
         <v>15</v>
       </c>
       <c r="F472">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G472">
         <v>0</v>
       </c>
       <c r="H472" t="str">
-        <v>26.7% (4/15戶)</v>
+        <v>33.3% (5/15戶)</v>
       </c>
       <c r="I472" t="str">
-        <v>26.7%</v>
+        <v>33.3%</v>
       </c>
       <c r="J472">
         <v>24.4</v>
@@ -35288,10 +35288,10 @@
         <v>24.4 ~ 24.5</v>
       </c>
       <c r="L472">
-        <v>1282</v>
+        <v>1281.6</v>
       </c>
       <c r="M472" t="str">
-        <v>115/04/04</v>
+        <v>115/08/02</v>
       </c>
       <c r="N472" t="str">
         <v>--</v>
@@ -35788,16 +35788,16 @@
         <v>8</v>
       </c>
       <c r="F479">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G479">
         <v>0</v>
       </c>
       <c r="H479" t="str">
-        <v>完銷 100%</v>
+        <v>87.5% (7/8戶)</v>
       </c>
       <c r="I479" t="str">
-        <v>100%</v>
+        <v>87.5%</v>
       </c>
       <c r="J479">
         <v>23.1</v>
@@ -35806,10 +35806,10 @@
         <v>21.7 ~ 25.9</v>
       </c>
       <c r="L479">
-        <v>1383.8</v>
+        <v>1384.3</v>
       </c>
       <c r="M479" t="str">
-        <v>115/07/25</v>
+        <v>114/10/11</v>
       </c>
       <c r="N479">
         <v>10.2</v>
@@ -36158,28 +36158,28 @@
         <v>65</v>
       </c>
       <c r="F484">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G484">
         <v>0</v>
       </c>
       <c r="H484" t="str">
-        <v>1.5% (1/65戶)</v>
+        <v>尚無實登</v>
       </c>
       <c r="I484" t="str">
-        <v>1.5%</v>
-      </c>
-      <c r="J484">
-        <v>36.3</v>
+        <v>尚無實登</v>
+      </c>
+      <c r="J484" t="str">
+        <v>--</v>
       </c>
       <c r="K484" t="str">
-        <v>36.3 ~ 36.3</v>
-      </c>
-      <c r="L484">
-        <v>1340</v>
+        <v>--</v>
+      </c>
+      <c r="L484" t="str">
+        <v>--</v>
       </c>
       <c r="M484" t="str">
-        <v>115/07/27</v>
+        <v>--</v>
       </c>
       <c r="N484" t="str">
         <v>--</v>
@@ -36602,28 +36602,28 @@
         <v>41</v>
       </c>
       <c r="F490">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="G490">
         <v>0</v>
       </c>
       <c r="H490" t="str">
-        <v>36.6% (15/41戶)</v>
+        <v>29.3% (12/41戶)</v>
       </c>
       <c r="I490" t="str">
-        <v>36.6%</v>
+        <v>29.3%</v>
       </c>
       <c r="J490">
-        <v>28.6</v>
+        <v>28.4</v>
       </c>
       <c r="K490" t="str">
         <v>25.9 ~ 33.2</v>
       </c>
       <c r="L490">
-        <v>1063.8</v>
+        <v>1047.1</v>
       </c>
       <c r="M490" t="str">
-        <v>115/07/30</v>
+        <v>115/04/29</v>
       </c>
       <c r="N490">
         <v>12</v>
@@ -36898,28 +36898,28 @@
         <v>34</v>
       </c>
       <c r="F494">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G494">
         <v>0</v>
       </c>
       <c r="H494" t="str">
-        <v>尚無實登</v>
+        <v>2.9% (1/34戶)</v>
       </c>
       <c r="I494" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J494" t="str">
-        <v>--</v>
+        <v>2.9%</v>
+      </c>
+      <c r="J494">
+        <v>23.9</v>
       </c>
       <c r="K494" t="str">
-        <v>--</v>
-      </c>
-      <c r="L494" t="str">
-        <v>--</v>
+        <v>23.9 ~ 23.9</v>
+      </c>
+      <c r="L494">
+        <v>545</v>
       </c>
       <c r="M494" t="str">
-        <v>--</v>
+        <v>115/08/03</v>
       </c>
       <c r="N494">
         <v>5</v>
@@ -37046,28 +37046,28 @@
         <v>24</v>
       </c>
       <c r="F496">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G496">
         <v>0</v>
       </c>
       <c r="H496" t="str">
-        <v>16.7% (4/24戶)</v>
+        <v>20.8% (5/24戶)</v>
       </c>
       <c r="I496" t="str">
-        <v>16.7%</v>
+        <v>20.8%</v>
       </c>
       <c r="J496">
-        <v>31.3</v>
+        <v>31.2</v>
       </c>
       <c r="K496" t="str">
         <v>30.8 ~ 31.8</v>
       </c>
       <c r="L496">
-        <v>1170.3</v>
+        <v>1128.8</v>
       </c>
       <c r="M496" t="str">
-        <v>114/12/18</v>
+        <v>115/08/06</v>
       </c>
       <c r="N496">
         <v>10</v>
@@ -37120,28 +37120,28 @@
         <v>30</v>
       </c>
       <c r="F497">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G497">
         <v>0</v>
       </c>
       <c r="H497" t="str">
-        <v>26.7% (8/30戶)</v>
+        <v>30% (9/30戶)</v>
       </c>
       <c r="I497" t="str">
-        <v>26.7%</v>
+        <v>30%</v>
       </c>
       <c r="J497">
-        <v>24.5</v>
+        <v>24.4</v>
       </c>
       <c r="K497" t="str">
         <v>22.8 ~ 26.2</v>
       </c>
       <c r="L497">
-        <v>1315.5</v>
+        <v>1301.3</v>
       </c>
       <c r="M497" t="str">
-        <v>115/01/20</v>
+        <v>115/08/03</v>
       </c>
       <c r="N497">
         <v>7.3</v>
@@ -37268,16 +37268,16 @@
         <v>65</v>
       </c>
       <c r="F499">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G499">
         <v>0</v>
       </c>
       <c r="H499" t="str">
-        <v>87.7% (57/65戶)</v>
+        <v>89.2% (58/65戶)</v>
       </c>
       <c r="I499" t="str">
-        <v>87.7%</v>
+        <v>89.2%</v>
       </c>
       <c r="J499">
         <v>26.8</v>
@@ -37286,10 +37286,10 @@
         <v>22.4 ~ 32</v>
       </c>
       <c r="L499">
-        <v>1003.2</v>
+        <v>1017.6</v>
       </c>
       <c r="M499" t="str">
-        <v>115/04/03</v>
+        <v>115/08/08</v>
       </c>
       <c r="N499" t="str">
         <v>--</v>
@@ -38082,16 +38082,16 @@
         <v>48</v>
       </c>
       <c r="F510">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G510">
         <v>0</v>
       </c>
       <c r="H510" t="str">
-        <v>14.6% (7/48戶)</v>
+        <v>12.5% (6/48戶)</v>
       </c>
       <c r="I510" t="str">
-        <v>14.6%</v>
+        <v>12.5%</v>
       </c>
       <c r="J510">
         <v>24.3</v>
@@ -38100,10 +38100,10 @@
         <v>22.5 ~ 29</v>
       </c>
       <c r="L510">
-        <v>789</v>
+        <v>789.2</v>
       </c>
       <c r="M510" t="str">
-        <v>115/07/25</v>
+        <v>115/04/07</v>
       </c>
       <c r="N510">
         <v>17.9</v>
@@ -38230,28 +38230,28 @@
         <v>24</v>
       </c>
       <c r="F512">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G512">
         <v>0</v>
       </c>
       <c r="H512" t="str">
-        <v>25% (6/24戶)</v>
+        <v>20.8% (5/24戶)</v>
       </c>
       <c r="I512" t="str">
-        <v>25%</v>
+        <v>20.8%</v>
       </c>
       <c r="J512">
-        <v>20.8</v>
+        <v>20.7</v>
       </c>
       <c r="K512" t="str">
         <v>19.6 ~ 22.4</v>
       </c>
       <c r="L512">
-        <v>508.7</v>
+        <v>506</v>
       </c>
       <c r="M512" t="str">
-        <v>115/07/25</v>
+        <v>115/04/15</v>
       </c>
       <c r="N512">
         <v>6.2</v>
@@ -38378,28 +38378,28 @@
         <v>16</v>
       </c>
       <c r="F514">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G514">
         <v>0</v>
       </c>
       <c r="H514" t="str">
-        <v>50% (8/16戶)</v>
+        <v>37.5% (6/16戶)</v>
       </c>
       <c r="I514" t="str">
-        <v>50%</v>
+        <v>37.5%</v>
       </c>
       <c r="J514">
-        <v>35.2</v>
+        <v>35.1</v>
       </c>
       <c r="K514" t="str">
-        <v>34.7 ~ 35.9</v>
+        <v>34.7 ~ 35.8</v>
       </c>
       <c r="L514">
-        <v>1933.6</v>
+        <v>1918.3</v>
       </c>
       <c r="M514" t="str">
-        <v>115/07/25</v>
+        <v>115/05/05</v>
       </c>
       <c r="N514" t="str">
         <v>--</v>
@@ -38470,10 +38470,10 @@
         <v>22.8 ~ 28.8</v>
       </c>
       <c r="L515">
-        <v>692.4</v>
+        <v>689.9</v>
       </c>
       <c r="M515" t="str">
-        <v>115/07/21</v>
+        <v>115/08/05</v>
       </c>
       <c r="N515">
         <v>5.3</v>
@@ -39266,28 +39266,28 @@
         <v>6</v>
       </c>
       <c r="F526">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G526">
         <v>0</v>
       </c>
       <c r="H526" t="str">
-        <v>16.7% (1/6戶)</v>
+        <v>尚無實登</v>
       </c>
       <c r="I526" t="str">
-        <v>16.7%</v>
-      </c>
-      <c r="J526">
-        <v>43</v>
+        <v>尚無實登</v>
+      </c>
+      <c r="J526" t="str">
+        <v>--</v>
       </c>
       <c r="K526" t="str">
-        <v>43 ~ 43</v>
-      </c>
-      <c r="L526">
-        <v>1315</v>
+        <v>--</v>
+      </c>
+      <c r="L526" t="str">
+        <v>--</v>
       </c>
       <c r="M526" t="str">
-        <v>115/07/23</v>
+        <v>--</v>
       </c>
       <c r="N526" t="str">
         <v>--</v>
@@ -39340,28 +39340,28 @@
         <v>22</v>
       </c>
       <c r="F527">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G527">
         <v>0</v>
       </c>
       <c r="H527" t="str">
-        <v>13.6% (3/22戶)</v>
+        <v>18.2% (4/22戶)</v>
       </c>
       <c r="I527" t="str">
-        <v>13.6%</v>
+        <v>18.2%</v>
       </c>
       <c r="J527">
-        <v>21.5</v>
+        <v>21.6</v>
       </c>
       <c r="K527" t="str">
         <v>20.7 ~ 22</v>
       </c>
       <c r="L527">
-        <v>634</v>
+        <v>678</v>
       </c>
       <c r="M527" t="str">
-        <v>115/03/25</v>
+        <v>115/08/05</v>
       </c>
       <c r="N527">
         <v>5.7</v>
@@ -39488,28 +39488,28 @@
         <v>25</v>
       </c>
       <c r="F529">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G529">
         <v>0</v>
       </c>
       <c r="H529" t="str">
-        <v>24% (6/25戶)</v>
+        <v>28% (7/25戶)</v>
       </c>
       <c r="I529" t="str">
-        <v>24%</v>
+        <v>28%</v>
       </c>
       <c r="J529">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="K529" t="str">
-        <v>21.8 ~ 23.3</v>
+        <v>21.8 ~ 23.5</v>
       </c>
       <c r="L529">
-        <v>1056.3</v>
+        <v>1055.1</v>
       </c>
       <c r="M529" t="str">
-        <v>115/04/24</v>
+        <v>115/08/04</v>
       </c>
       <c r="N529" t="str">
         <v>--</v>
@@ -39722,16 +39722,16 @@
         <v>14%</v>
       </c>
       <c r="J532">
-        <v>21.6</v>
+        <v>21.5</v>
       </c>
       <c r="K532" t="str">
         <v>19.4 ~ 22.6</v>
       </c>
       <c r="L532">
-        <v>767.1</v>
+        <v>760</v>
       </c>
       <c r="M532" t="str">
-        <v>115/07/26</v>
+        <v>115/08/02</v>
       </c>
       <c r="N532">
         <v>8.6</v>
@@ -40820,28 +40820,28 @@
         <v>28</v>
       </c>
       <c r="F547">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G547">
         <v>0</v>
       </c>
       <c r="H547" t="str">
-        <v>尚無實登</v>
+        <v>25% (7/28戶)</v>
       </c>
       <c r="I547" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J547" t="str">
-        <v>--</v>
+        <v>25%</v>
+      </c>
+      <c r="J547">
+        <v>31.7</v>
       </c>
       <c r="K547" t="str">
-        <v>--</v>
-      </c>
-      <c r="L547" t="str">
-        <v>--</v>
+        <v>28.5 ~ 34.9</v>
+      </c>
+      <c r="L547">
+        <v>871.6</v>
       </c>
       <c r="M547" t="str">
-        <v>--</v>
+        <v>115/08/01</v>
       </c>
       <c r="N547">
         <v>11</v>
@@ -40894,28 +40894,28 @@
         <v>16</v>
       </c>
       <c r="F548">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G548">
         <v>0</v>
       </c>
       <c r="H548" t="str">
-        <v>尚無實登</v>
+        <v>6.3% (1/16戶)</v>
       </c>
       <c r="I548" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J548" t="str">
-        <v>--</v>
+        <v>6.3%</v>
+      </c>
+      <c r="J548">
+        <v>26.9</v>
       </c>
       <c r="K548" t="str">
-        <v>--</v>
-      </c>
-      <c r="L548" t="str">
-        <v>--</v>
+        <v>26.9 ~ 26.9</v>
+      </c>
+      <c r="L548">
+        <v>850</v>
       </c>
       <c r="M548" t="str">
-        <v>--</v>
+        <v>115/08/08</v>
       </c>
       <c r="N548">
         <v>9.7</v>
@@ -41116,28 +41116,28 @@
         <v>24</v>
       </c>
       <c r="F551">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G551">
         <v>0</v>
       </c>
       <c r="H551" t="str">
-        <v>4.2% (1/24戶)</v>
+        <v>尚無實登</v>
       </c>
       <c r="I551" t="str">
-        <v>4.2%</v>
-      </c>
-      <c r="J551">
-        <v>25.5</v>
+        <v>尚無實登</v>
+      </c>
+      <c r="J551" t="str">
+        <v>--</v>
       </c>
       <c r="K551" t="str">
-        <v>25.5 ~ 25.5</v>
-      </c>
-      <c r="L551">
-        <v>399</v>
+        <v>--</v>
+      </c>
+      <c r="L551" t="str">
+        <v>--</v>
       </c>
       <c r="M551" t="str">
-        <v>115/07/25</v>
+        <v>--</v>
       </c>
       <c r="N551">
         <v>15</v>
@@ -41338,28 +41338,28 @@
         <v>8</v>
       </c>
       <c r="F554">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G554">
         <v>0</v>
       </c>
       <c r="H554" t="str">
-        <v>12.5% (1/8戶)</v>
+        <v>尚無實登</v>
       </c>
       <c r="I554" t="str">
-        <v>12.5%</v>
-      </c>
-      <c r="J554">
-        <v>23.2</v>
+        <v>尚無實登</v>
+      </c>
+      <c r="J554" t="str">
+        <v>--</v>
       </c>
       <c r="K554" t="str">
-        <v>23.2 ~ 23.2</v>
-      </c>
-      <c r="L554">
-        <v>998</v>
+        <v>--</v>
+      </c>
+      <c r="L554" t="str">
+        <v>--</v>
       </c>
       <c r="M554" t="str">
-        <v>115/07/24</v>
+        <v>--</v>
       </c>
       <c r="N554">
         <v>13.4</v>
@@ -41486,28 +41486,28 @@
         <v>17</v>
       </c>
       <c r="F556">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G556">
         <v>0</v>
       </c>
       <c r="H556" t="str">
-        <v>5.9% (1/17戶)</v>
+        <v>尚無實登</v>
       </c>
       <c r="I556" t="str">
-        <v>5.9%</v>
-      </c>
-      <c r="J556">
-        <v>30.9</v>
+        <v>尚無實登</v>
+      </c>
+      <c r="J556" t="str">
+        <v>--</v>
       </c>
       <c r="K556" t="str">
-        <v>30.9 ~ 30.9</v>
-      </c>
-      <c r="L556">
-        <v>708</v>
+        <v>--</v>
+      </c>
+      <c r="L556" t="str">
+        <v>--</v>
       </c>
       <c r="M556" t="str">
-        <v>115/07/30</v>
+        <v>--</v>
       </c>
       <c r="N556">
         <v>21.2</v>
@@ -41572,16 +41572,16 @@
         <v>5.3%</v>
       </c>
       <c r="J557">
-        <v>27.1</v>
+        <v>26.5</v>
       </c>
       <c r="K557" t="str">
-        <v>27.1 ~ 27.1</v>
+        <v>26.5 ~ 26.5</v>
       </c>
       <c r="L557">
-        <v>1428</v>
+        <v>1398</v>
       </c>
       <c r="M557" t="str">
-        <v>115/07/27</v>
+        <v>115/08/05</v>
       </c>
       <c r="N557">
         <v>10.8</v>
@@ -41782,28 +41782,28 @@
         <v>31</v>
       </c>
       <c r="F560">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G560">
         <v>0</v>
       </c>
       <c r="H560" t="str">
-        <v>6.5% (2/31戶)</v>
+        <v>尚無實登</v>
       </c>
       <c r="I560" t="str">
-        <v>6.5%</v>
-      </c>
-      <c r="J560">
-        <v>23.9</v>
+        <v>尚無實登</v>
+      </c>
+      <c r="J560" t="str">
+        <v>--</v>
       </c>
       <c r="K560" t="str">
-        <v>23 ~ 24.7</v>
-      </c>
-      <c r="L560">
-        <v>1315</v>
+        <v>--</v>
+      </c>
+      <c r="L560" t="str">
+        <v>--</v>
       </c>
       <c r="M560" t="str">
-        <v>115/07/27</v>
+        <v>--</v>
       </c>
       <c r="N560">
         <v>12</v>
@@ -41856,28 +41856,28 @@
         <v>32</v>
       </c>
       <c r="F561">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G561">
         <v>0</v>
       </c>
       <c r="H561" t="str">
-        <v>尚無實登</v>
+        <v>15.6% (5/32戶)</v>
       </c>
       <c r="I561" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J561" t="str">
-        <v>--</v>
+        <v>15.6%</v>
+      </c>
+      <c r="J561">
+        <v>28.8</v>
       </c>
       <c r="K561" t="str">
-        <v>--</v>
-      </c>
-      <c r="L561" t="str">
-        <v>--</v>
+        <v>26.2 ~ 30.6</v>
+      </c>
+      <c r="L561">
+        <v>591.2</v>
       </c>
       <c r="M561" t="str">
-        <v>--</v>
+        <v>115/08/09</v>
       </c>
       <c r="N561">
         <v>12.6</v>
@@ -41930,28 +41930,28 @@
         <v>42</v>
       </c>
       <c r="F562">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G562">
         <v>0</v>
       </c>
       <c r="H562" t="str">
-        <v>11.9% (5/42戶)</v>
+        <v>7.1% (3/42戶)</v>
       </c>
       <c r="I562" t="str">
-        <v>11.9%</v>
+        <v>7.1%</v>
       </c>
       <c r="J562">
-        <v>28.8</v>
+        <v>30.2</v>
       </c>
       <c r="K562" t="str">
-        <v>28 ~ 29.3</v>
+        <v>28.9 ~ 32.3</v>
       </c>
       <c r="L562">
-        <v>677.6</v>
+        <v>1001.7</v>
       </c>
       <c r="M562" t="str">
-        <v>115/07/31</v>
+        <v>115/08/08</v>
       </c>
       <c r="N562">
         <v>10</v>
@@ -42152,28 +42152,28 @@
         <v>11</v>
       </c>
       <c r="F565">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G565">
         <v>0</v>
       </c>
       <c r="H565" t="str">
-        <v>9.1% (1/11戶)</v>
+        <v>尚無實登</v>
       </c>
       <c r="I565" t="str">
-        <v>9.1%</v>
-      </c>
-      <c r="J565">
-        <v>34.1</v>
+        <v>尚無實登</v>
+      </c>
+      <c r="J565" t="str">
+        <v>--</v>
       </c>
       <c r="K565" t="str">
-        <v>34.1 ~ 34.1</v>
-      </c>
-      <c r="L565">
-        <v>988</v>
+        <v>--</v>
+      </c>
+      <c r="L565" t="str">
+        <v>--</v>
       </c>
       <c r="M565" t="str">
-        <v>115/07/29</v>
+        <v>--</v>
       </c>
       <c r="N565" t="str">
         <v>--</v>
@@ -42682,16 +42682,16 @@
         <v>15.4%</v>
       </c>
       <c r="J572">
-        <v>24.3</v>
+        <v>24.4</v>
       </c>
       <c r="K572" t="str">
-        <v>23.5 ~ 25.1</v>
+        <v>23.8 ~ 25</v>
       </c>
       <c r="L572">
-        <v>1343</v>
+        <v>1168</v>
       </c>
       <c r="M572" t="str">
-        <v>115/07/31</v>
+        <v>115/08/09</v>
       </c>
       <c r="N572">
         <v>14.5</v>
@@ -43040,28 +43040,28 @@
         <v>22</v>
       </c>
       <c r="F577">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G577">
         <v>0</v>
       </c>
       <c r="H577" t="str">
-        <v>尚無實登</v>
+        <v>4.5% (1/22戶)</v>
       </c>
       <c r="I577" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J577" t="str">
-        <v>--</v>
+        <v>4.5%</v>
+      </c>
+      <c r="J577">
+        <v>30</v>
       </c>
       <c r="K577" t="str">
-        <v>--</v>
-      </c>
-      <c r="L577" t="str">
-        <v>--</v>
+        <v>30 ~ 30</v>
+      </c>
+      <c r="L577">
+        <v>656</v>
       </c>
       <c r="M577" t="str">
-        <v>--</v>
+        <v>115/08/10</v>
       </c>
       <c r="N577">
         <v>6.7</v>
@@ -43188,28 +43188,28 @@
         <v>15</v>
       </c>
       <c r="F579">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G579">
         <v>0</v>
       </c>
       <c r="H579" t="str">
-        <v>20% (3/15戶)</v>
+        <v>尚無實登</v>
       </c>
       <c r="I579" t="str">
-        <v>20%</v>
-      </c>
-      <c r="J579">
-        <v>27.5</v>
+        <v>尚無實登</v>
+      </c>
+      <c r="J579" t="str">
+        <v>--</v>
       </c>
       <c r="K579" t="str">
-        <v>25.4 ~ 28.7</v>
-      </c>
-      <c r="L579">
-        <v>653.3</v>
+        <v>--</v>
+      </c>
+      <c r="L579" t="str">
+        <v>--</v>
       </c>
       <c r="M579" t="str">
-        <v>115/07/31</v>
+        <v>--</v>
       </c>
       <c r="N579" t="str">
         <v>--</v>

</xml_diff>

<commit_message>
fix: normalize NO. prefixes and dots in matching to include 美澍家NO.10 transactions
</commit_message>
<xml_diff>
--- a/宜蘭建案實價登錄銷售統計.xlsx
+++ b/宜蘭建案實價登錄銷售統計.xlsx
@@ -8790,13 +8790,13 @@
         <v>100%</v>
       </c>
       <c r="J114">
-        <v>30.3</v>
+        <v>30</v>
       </c>
       <c r="K114" t="str">
-        <v>29.9 ~ 31.1</v>
+        <v>28.8 ~ 31.1</v>
       </c>
       <c r="L114">
-        <v>1763.3</v>
+        <v>1851.3</v>
       </c>
       <c r="M114" t="str">
         <v>112/06/29</v>
@@ -28314,19 +28314,19 @@
         <v>7</v>
       </c>
       <c r="F378">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G378">
         <v>0</v>
       </c>
       <c r="H378" t="str">
-        <v>28.6% (2/7戶)</v>
+        <v>42.9% (3/7戶)</v>
       </c>
       <c r="I378" t="str">
-        <v>28.6%</v>
+        <v>42.9%</v>
       </c>
       <c r="J378">
-        <v>23.5</v>
+        <v>23.4</v>
       </c>
       <c r="K378" t="str">
         <v>23.1 ~ 23.9</v>
@@ -28335,7 +28335,7 @@
         <v>1680</v>
       </c>
       <c r="M378" t="str">
-        <v>114/01/10</v>
+        <v>114/01/14</v>
       </c>
       <c r="N378">
         <v>9.6</v>
@@ -32162,25 +32162,25 @@
         <v>7</v>
       </c>
       <c r="F430">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G430">
         <v>0</v>
       </c>
       <c r="H430" t="str">
-        <v>42.9% (3/7戶)</v>
+        <v>57.1% (4/7戶)</v>
       </c>
       <c r="I430" t="str">
-        <v>42.9%</v>
+        <v>57.1%</v>
       </c>
       <c r="J430">
-        <v>41.6</v>
+        <v>41.5</v>
       </c>
       <c r="K430" t="str">
-        <v>41.1 ~ 42.3</v>
+        <v>41 ~ 42.3</v>
       </c>
       <c r="L430">
-        <v>2713.3</v>
+        <v>2692.5</v>
       </c>
       <c r="M430" t="str">
         <v>114/12/30</v>
@@ -38896,28 +38896,28 @@
         <v>38</v>
       </c>
       <c r="F521">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="G521">
         <v>0</v>
       </c>
       <c r="H521" t="str">
-        <v>尚無實登</v>
+        <v>15.8% (6/38戶)</v>
       </c>
       <c r="I521" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J521" t="str">
-        <v>--</v>
+        <v>15.8%</v>
+      </c>
+      <c r="J521">
+        <v>35.7</v>
       </c>
       <c r="K521" t="str">
-        <v>--</v>
-      </c>
-      <c r="L521" t="str">
-        <v>--</v>
+        <v>34.2 ~ 36.7</v>
+      </c>
+      <c r="L521">
+        <v>1430.8</v>
       </c>
       <c r="M521" t="str">
-        <v>--</v>
+        <v>115/08/10</v>
       </c>
       <c r="N521" t="str">
         <v>--</v>

</xml_diff>

<commit_message>
fix: comprehensive symbol normalization and Big5 question mark wildcard matching (recovering 292 missed units across 16 projects)
</commit_message>
<xml_diff>
--- a/宜蘭建案實價登錄銷售統計.xlsx
+++ b/宜蘭建案實價登錄銷售統計.xlsx
@@ -3154,28 +3154,28 @@
         <v>20</v>
       </c>
       <c r="F38">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G38">
         <v>0</v>
       </c>
       <c r="H38" t="str">
-        <v>尚無實登</v>
+        <v>90% (18/20戶)</v>
       </c>
       <c r="I38" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J38" t="str">
-        <v>--</v>
+        <v>90%</v>
+      </c>
+      <c r="J38">
+        <v>22.3</v>
       </c>
       <c r="K38" t="str">
-        <v>--</v>
-      </c>
-      <c r="L38" t="str">
-        <v>--</v>
+        <v>20 ~ 23</v>
+      </c>
+      <c r="L38">
+        <v>1866.1</v>
       </c>
       <c r="M38" t="str">
-        <v>--</v>
+        <v>112/04/15</v>
       </c>
       <c r="N38">
         <v>7</v>
@@ -4190,28 +4190,28 @@
         <v>32</v>
       </c>
       <c r="F52">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="G52">
         <v>0</v>
       </c>
       <c r="H52" t="str">
-        <v>尚無實登</v>
+        <v>96.9% (31/32戶)</v>
       </c>
       <c r="I52" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J52" t="str">
-        <v>--</v>
+        <v>96.9%</v>
+      </c>
+      <c r="J52">
+        <v>22.1</v>
       </c>
       <c r="K52" t="str">
-        <v>--</v>
-      </c>
-      <c r="L52" t="str">
-        <v>--</v>
+        <v>20.9 ~ 26.3</v>
+      </c>
+      <c r="L52">
+        <v>636</v>
       </c>
       <c r="M52" t="str">
-        <v>--</v>
+        <v>111/07/29</v>
       </c>
       <c r="N52">
         <v>14.7</v>
@@ -6558,28 +6558,28 @@
         <v>20</v>
       </c>
       <c r="F84">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="G84">
         <v>0</v>
       </c>
       <c r="H84" t="str">
-        <v>尚無實登</v>
+        <v>完銷 100%</v>
       </c>
       <c r="I84" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J84" t="str">
-        <v>--</v>
+        <v>100%</v>
+      </c>
+      <c r="J84">
+        <v>16.9</v>
       </c>
       <c r="K84" t="str">
-        <v>--</v>
-      </c>
-      <c r="L84" t="str">
-        <v>--</v>
+        <v>16.7 ~ 17.7</v>
+      </c>
+      <c r="L84">
+        <v>422.9</v>
       </c>
       <c r="M84" t="str">
-        <v>--</v>
+        <v>113/04/15</v>
       </c>
       <c r="N84" t="str">
         <v>--</v>
@@ -8556,28 +8556,28 @@
         <v>13</v>
       </c>
       <c r="F111">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G111">
         <v>0</v>
       </c>
       <c r="H111" t="str">
-        <v>尚無實登</v>
+        <v>92.3% (12/13戶)</v>
       </c>
       <c r="I111" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J111" t="str">
-        <v>--</v>
+        <v>92.3%</v>
+      </c>
+      <c r="J111">
+        <v>18.2</v>
       </c>
       <c r="K111" t="str">
-        <v>--</v>
-      </c>
-      <c r="L111" t="str">
-        <v>--</v>
+        <v>17.3 ~ 19.6</v>
+      </c>
+      <c r="L111">
+        <v>839.8</v>
       </c>
       <c r="M111" t="str">
-        <v>--</v>
+        <v>111/10/15</v>
       </c>
       <c r="N111" t="str">
         <v>--</v>
@@ -9740,28 +9740,28 @@
         <v>45</v>
       </c>
       <c r="F127">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="G127">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H127" t="str">
-        <v>尚無實登</v>
+        <v>93.3% (42/45戶)</v>
       </c>
       <c r="I127" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J127" t="str">
-        <v>--</v>
+        <v>93.3%</v>
+      </c>
+      <c r="J127">
+        <v>34.3</v>
       </c>
       <c r="K127" t="str">
-        <v>--</v>
-      </c>
-      <c r="L127" t="str">
-        <v>--</v>
+        <v>31.5 ~ 38.9</v>
+      </c>
+      <c r="L127">
+        <v>1289.5</v>
       </c>
       <c r="M127" t="str">
-        <v>--</v>
+        <v>113/11/05</v>
       </c>
       <c r="N127" t="str">
         <v>--</v>
@@ -13366,28 +13366,28 @@
         <v>21</v>
       </c>
       <c r="F176">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="G176">
         <v>0</v>
       </c>
       <c r="H176" t="str">
-        <v>尚無實登</v>
+        <v>85.7% (18/21戶)</v>
       </c>
       <c r="I176" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J176" t="str">
-        <v>--</v>
+        <v>85.7%</v>
+      </c>
+      <c r="J176">
+        <v>24.8</v>
       </c>
       <c r="K176" t="str">
-        <v>--</v>
-      </c>
-      <c r="L176" t="str">
-        <v>--</v>
+        <v>23.5 ~ 26.7</v>
+      </c>
+      <c r="L176">
+        <v>700.3</v>
       </c>
       <c r="M176" t="str">
-        <v>--</v>
+        <v>114/09/17</v>
       </c>
       <c r="N176" t="str">
         <v>--</v>
@@ -14328,28 +14328,28 @@
         <v>36</v>
       </c>
       <c r="F189">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="G189">
         <v>0</v>
       </c>
       <c r="H189" t="str">
-        <v>尚無實登</v>
+        <v>完銷 100%</v>
       </c>
       <c r="I189" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J189" t="str">
-        <v>--</v>
+        <v>100%</v>
+      </c>
+      <c r="J189">
+        <v>25.7</v>
       </c>
       <c r="K189" t="str">
-        <v>--</v>
-      </c>
-      <c r="L189" t="str">
-        <v>--</v>
+        <v>23.5 ~ 31.7</v>
+      </c>
+      <c r="L189">
+        <v>758.7</v>
       </c>
       <c r="M189" t="str">
-        <v>--</v>
+        <v>112/11/25</v>
       </c>
       <c r="N189">
         <v>16.8</v>
@@ -16548,28 +16548,28 @@
         <v>24</v>
       </c>
       <c r="F219">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="G219">
         <v>0</v>
       </c>
       <c r="H219" t="str">
-        <v>尚無實登</v>
+        <v>完銷 100%</v>
       </c>
       <c r="I219" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J219" t="str">
-        <v>--</v>
+        <v>100%</v>
+      </c>
+      <c r="J219">
+        <v>17.9</v>
       </c>
       <c r="K219" t="str">
-        <v>--</v>
-      </c>
-      <c r="L219" t="str">
-        <v>--</v>
+        <v>17.1 ~ 19.2</v>
+      </c>
+      <c r="L219">
+        <v>476.5</v>
       </c>
       <c r="M219" t="str">
-        <v>--</v>
+        <v>112/09/28</v>
       </c>
       <c r="N219">
         <v>6.5</v>
@@ -22320,28 +22320,28 @@
         <v>22</v>
       </c>
       <c r="F297">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="G297">
         <v>0</v>
       </c>
       <c r="H297" t="str">
-        <v>尚無實登</v>
+        <v>完銷 100%</v>
       </c>
       <c r="I297" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J297" t="str">
-        <v>--</v>
+        <v>100%</v>
+      </c>
+      <c r="J297">
+        <v>33.3</v>
       </c>
       <c r="K297" t="str">
-        <v>--</v>
-      </c>
-      <c r="L297" t="str">
-        <v>--</v>
+        <v>28.5 ~ 40.3</v>
+      </c>
+      <c r="L297">
+        <v>940</v>
       </c>
       <c r="M297" t="str">
-        <v>--</v>
+        <v>114/11/03</v>
       </c>
       <c r="N297">
         <v>16.9</v>
@@ -25798,28 +25798,28 @@
         <v>21</v>
       </c>
       <c r="F344">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="G344">
         <v>0</v>
       </c>
       <c r="H344" t="str">
-        <v>尚無實登</v>
+        <v>90.5% (19/21戶)</v>
       </c>
       <c r="I344" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J344" t="str">
-        <v>--</v>
+        <v>90.5%</v>
+      </c>
+      <c r="J344">
+        <v>19.8</v>
       </c>
       <c r="K344" t="str">
-        <v>--</v>
-      </c>
-      <c r="L344" t="str">
-        <v>--</v>
+        <v>18.7 ~ 21.3</v>
+      </c>
+      <c r="L344">
+        <v>587</v>
       </c>
       <c r="M344" t="str">
-        <v>--</v>
+        <v>115/03/06</v>
       </c>
       <c r="N344">
         <v>10</v>
@@ -30016,28 +30016,28 @@
         <v>5</v>
       </c>
       <c r="F401">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G401">
         <v>0</v>
       </c>
       <c r="H401" t="str">
-        <v>尚無實登</v>
+        <v>60% (3/5戶)</v>
       </c>
       <c r="I401" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J401" t="str">
-        <v>--</v>
+        <v>60%</v>
+      </c>
+      <c r="J401">
+        <v>32.8</v>
       </c>
       <c r="K401" t="str">
-        <v>--</v>
-      </c>
-      <c r="L401" t="str">
-        <v>--</v>
+        <v>32 ~ 34</v>
+      </c>
+      <c r="L401">
+        <v>1858.7</v>
       </c>
       <c r="M401" t="str">
-        <v>--</v>
+        <v>114/01/16</v>
       </c>
       <c r="N401" t="str">
         <v>--</v>
@@ -30090,28 +30090,28 @@
         <v>30</v>
       </c>
       <c r="F402">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="G402">
         <v>0</v>
       </c>
       <c r="H402" t="str">
-        <v>尚無實登</v>
+        <v>83.3% (25/30戶)</v>
       </c>
       <c r="I402" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J402" t="str">
-        <v>--</v>
+        <v>83.3%</v>
+      </c>
+      <c r="J402">
+        <v>34</v>
       </c>
       <c r="K402" t="str">
-        <v>--</v>
-      </c>
-      <c r="L402" t="str">
-        <v>--</v>
+        <v>30.9 ~ 36.7</v>
+      </c>
+      <c r="L402">
+        <v>1095.7</v>
       </c>
       <c r="M402" t="str">
-        <v>--</v>
+        <v>115/04/08</v>
       </c>
       <c r="N402" t="str">
         <v>--</v>
@@ -34086,25 +34086,25 @@
         <v>36</v>
       </c>
       <c r="F456">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="G456">
         <v>0</v>
       </c>
       <c r="H456" t="str">
-        <v>2.8% (1/36戶)</v>
+        <v>61.1% (22/36戶)</v>
       </c>
       <c r="I456" t="str">
-        <v>2.8%</v>
+        <v>61.1%</v>
       </c>
       <c r="J456">
-        <v>25.8</v>
+        <v>24.8</v>
       </c>
       <c r="K456" t="str">
-        <v>25.8 ~ 25.8</v>
+        <v>21.3 ~ 29.9</v>
       </c>
       <c r="L456">
-        <v>868</v>
+        <v>726.6</v>
       </c>
       <c r="M456" t="str">
         <v>115/07/12</v>
@@ -38970,28 +38970,28 @@
         <v>4</v>
       </c>
       <c r="F522">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G522">
         <v>0</v>
       </c>
       <c r="H522" t="str">
-        <v>尚無實登</v>
+        <v>25% (1/4戶)</v>
       </c>
       <c r="I522" t="str">
-        <v>尚無實登</v>
-      </c>
-      <c r="J522" t="str">
-        <v>--</v>
+        <v>25%</v>
+      </c>
+      <c r="J522">
+        <v>29.8</v>
       </c>
       <c r="K522" t="str">
-        <v>--</v>
-      </c>
-      <c r="L522" t="str">
-        <v>--</v>
+        <v>29.8 ~ 29.8</v>
+      </c>
+      <c r="L522">
+        <v>2200</v>
       </c>
       <c r="M522" t="str">
-        <v>--</v>
+        <v>115/04/30</v>
       </c>
       <c r="N522" t="str">
         <v>--</v>

</xml_diff>

<commit_message>
Schedule update: adjust to 1st, 11th, 21st (morning 10:30 & afternoon 15:30) with smart change detection
</commit_message>
<xml_diff>
--- a/宜蘭建案實價登錄銷售統計.xlsx
+++ b/宜蘭建案實價登錄銷售統計.xlsx
@@ -32680,28 +32680,28 @@
         <v>25</v>
       </c>
       <c r="F437">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G437">
         <v>0</v>
       </c>
       <c r="H437" t="str">
-        <v>52% (13/25戶)</v>
+        <v>56% (14/25戶)</v>
       </c>
       <c r="I437" t="str">
-        <v>52%</v>
+        <v>56%</v>
       </c>
       <c r="J437">
-        <v>31.3</v>
+        <v>31.2</v>
       </c>
       <c r="K437" t="str">
         <v>28 ~ 45</v>
       </c>
       <c r="L437">
-        <v>1368</v>
+        <v>1362.1</v>
       </c>
       <c r="M437" t="str">
-        <v>115/05/23</v>
+        <v>115/08/05</v>
       </c>
       <c r="N437">
         <v>9.6</v>

</xml_diff>